<commit_message>
simulasi_asn_rev: hyperlinks between related tables and sheets
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QL8Do8Pd2rXEDNa1ifG2RK
</commit_message>
<xml_diff>
--- a/deliverables/simulasi_asn_rev.xlsx
+++ b/deliverables/simulasi_asn_rev.xlsx
@@ -17,11 +17,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -75,6 +74,16 @@
     </font>
     <font>
       <i val="1"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="FF0563C1"/>
+      <sz val="8"/>
+      <u val="single"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="FF0563C1"/>
     </font>
   </fonts>
   <fills count="14">
@@ -204,7 +213,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="62">
+  <cellXfs count="69">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -351,16 +360,35 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="5" fillId="11" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="5" fillId="11" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="13" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="13" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="5" fillId="13" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="11" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="11" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="13" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="13" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -704,7 +732,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N133"/>
+  <dimension ref="A1:N134"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="13.90625" customWidth="1" style="26" min="1" max="1"/>
@@ -803,7 +831,7 @@
           <t>9715300</t>
         </is>
       </c>
-      <c r="B5" s="13" t="inlineStr">
+      <c r="B5" s="62" t="inlineStr">
         <is>
           <t>CO-14101</t>
         </is>
@@ -854,7 +882,7 @@
           <t>9722D10</t>
         </is>
       </c>
-      <c r="B6" s="13" t="inlineStr">
+      <c r="B6" s="62" t="inlineStr">
         <is>
           <t>CO-14102</t>
         </is>
@@ -900,6 +928,7 @@
       </c>
     </row>
     <row r="7" customFormat="1" s="20"/>
+    <row r="8"/>
     <row r="9" s="26">
       <c r="A9" s="39" t="inlineStr">
         <is>
@@ -1273,7 +1302,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M21" s="56" t="inlineStr">
+      <c r="M21" s="63" t="inlineStr">
         <is>
           <t>ASN0001</t>
         </is>
@@ -1437,7 +1466,7 @@
           <t>9715300</t>
         </is>
       </c>
-      <c r="B29" s="13" t="inlineStr">
+      <c r="B29" s="62" t="inlineStr">
         <is>
           <t>CO-14101</t>
         </is>
@@ -1484,7 +1513,7 @@
           <t>9722D10</t>
         </is>
       </c>
-      <c r="B30" s="13" t="inlineStr">
+      <c r="B30" s="62" t="inlineStr">
         <is>
           <t>CO-14102</t>
         </is>
@@ -1531,7 +1560,7 @@
           <t>9722D10</t>
         </is>
       </c>
-      <c r="B31" s="13" t="inlineStr">
+      <c r="B31" s="62" t="inlineStr">
         <is>
           <t>CO-14103</t>
         </is>
@@ -1724,7 +1753,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M38" s="13" t="inlineStr">
+      <c r="M38" s="62" t="inlineStr">
         <is>
           <t>ASN0001</t>
         </is>
@@ -1872,6 +1901,7 @@
       </c>
     </row>
     <row r="41" ht="21" customHeight="1" s="26"/>
+    <row r="42"/>
     <row r="43">
       <c r="A43" s="39" t="inlineStr">
         <is>
@@ -2022,7 +2052,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M47" s="13" t="inlineStr">
+      <c r="M47" s="62" t="inlineStr">
         <is>
           <t>ASN0001</t>
         </is>
@@ -2158,7 +2188,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M49" s="56" t="inlineStr">
+      <c r="M49" s="63" t="inlineStr">
         <is>
           <t>ASN0002</t>
         </is>
@@ -2170,6 +2200,7 @@
       </c>
     </row>
     <row r="50" ht="21" customHeight="1" s="26"/>
+    <row r="51"/>
     <row r="52">
       <c r="A52" s="39" t="inlineStr">
         <is>
@@ -2253,7 +2284,7 @@
           <t>9715300</t>
         </is>
       </c>
-      <c r="B56" s="13" t="inlineStr">
+      <c r="B56" s="62" t="inlineStr">
         <is>
           <t>CO-14101</t>
         </is>
@@ -2300,7 +2331,7 @@
           <t>9722D10</t>
         </is>
       </c>
-      <c r="B57" s="13" t="inlineStr">
+      <c r="B57" s="62" t="inlineStr">
         <is>
           <t>CO-14102</t>
         </is>
@@ -2347,7 +2378,7 @@
           <t>9722D10</t>
         </is>
       </c>
-      <c r="B58" s="13" t="inlineStr">
+      <c r="B58" s="62" t="inlineStr">
         <is>
           <t>CO-14103</t>
         </is>
@@ -2394,7 +2425,7 @@
           <t>9722D10</t>
         </is>
       </c>
-      <c r="B59" s="13" t="inlineStr">
+      <c r="B59" s="62" t="inlineStr">
         <is>
           <t>CO-14104</t>
         </is>
@@ -2441,7 +2472,7 @@
           <t>9715300</t>
         </is>
       </c>
-      <c r="B60" s="13" t="inlineStr">
+      <c r="B60" s="62" t="inlineStr">
         <is>
           <t>CO-14105</t>
         </is>
@@ -2488,7 +2519,7 @@
           <t>9715300</t>
         </is>
       </c>
-      <c r="B61" s="13" t="inlineStr">
+      <c r="B61" s="62" t="inlineStr">
         <is>
           <t>CO-14106</t>
         </is>
@@ -2535,7 +2566,7 @@
           <t>9715300</t>
         </is>
       </c>
-      <c r="B62" s="13" t="inlineStr">
+      <c r="B62" s="62" t="inlineStr">
         <is>
           <t>CO-14107</t>
         </is>
@@ -2582,7 +2613,7 @@
           <t>9722D10</t>
         </is>
       </c>
-      <c r="B63" s="13" t="inlineStr">
+      <c r="B63" s="62" t="inlineStr">
         <is>
           <t>CO-14108</t>
         </is>
@@ -2627,6 +2658,7 @@
         </is>
       </c>
     </row>
+    <row r="64"/>
     <row r="65" customFormat="1" s="30"/>
     <row r="66" customFormat="1" s="34">
       <c r="A66" s="39" t="inlineStr">
@@ -2778,7 +2810,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M70" s="13" t="inlineStr">
+      <c r="M70" s="62" t="inlineStr">
         <is>
           <t>ASN0001</t>
         </is>
@@ -2914,7 +2946,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M72" s="13" t="inlineStr">
+      <c r="M72" s="62" t="inlineStr">
         <is>
           <t>ASN0002</t>
         </is>
@@ -3265,6 +3297,8 @@
         </is>
       </c>
     </row>
+    <row r="78"/>
+    <row r="79"/>
     <row r="80" customFormat="1" s="34">
       <c r="A80" s="39" t="inlineStr">
         <is>
@@ -3415,7 +3449,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M84" s="13" t="inlineStr">
+      <c r="M84" s="62" t="inlineStr">
         <is>
           <t>ASN0001</t>
         </is>
@@ -3551,7 +3585,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M86" s="13" t="inlineStr">
+      <c r="M86" s="62" t="inlineStr">
         <is>
           <t>ASN0002</t>
         </is>
@@ -3619,7 +3653,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M87" s="56" t="inlineStr">
+      <c r="M87" s="63" t="inlineStr">
         <is>
           <t>ASN0003</t>
         </is>
@@ -3687,7 +3721,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M88" s="56" t="inlineStr">
+      <c r="M88" s="63" t="inlineStr">
         <is>
           <t>ASN0003</t>
         </is>
@@ -3755,7 +3789,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M89" s="56" t="inlineStr">
+      <c r="M89" s="63" t="inlineStr">
         <is>
           <t>ASN0003</t>
         </is>
@@ -3823,7 +3857,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M90" s="56" t="inlineStr">
+      <c r="M90" s="63" t="inlineStr">
         <is>
           <t>ASN0003</t>
         </is>
@@ -3903,6 +3937,7 @@
       </c>
     </row>
     <row r="92" ht="15" customHeight="1" s="26"/>
+    <row r="93"/>
     <row r="94">
       <c r="A94" s="39" t="inlineStr">
         <is>
@@ -3986,7 +4021,7 @@
           <t>9715300</t>
         </is>
       </c>
-      <c r="B98" s="13" t="inlineStr">
+      <c r="B98" s="62" t="inlineStr">
         <is>
           <t>CO-14101</t>
         </is>
@@ -4033,7 +4068,7 @@
           <t>9722D10</t>
         </is>
       </c>
-      <c r="B99" s="13" t="inlineStr">
+      <c r="B99" s="62" t="inlineStr">
         <is>
           <t>CO-14102</t>
         </is>
@@ -4080,7 +4115,7 @@
           <t>9722D10</t>
         </is>
       </c>
-      <c r="B100" s="13" t="inlineStr">
+      <c r="B100" s="62" t="inlineStr">
         <is>
           <t>CO-14103</t>
         </is>
@@ -4127,7 +4162,7 @@
           <t>9722D10</t>
         </is>
       </c>
-      <c r="B101" s="13" t="inlineStr">
+      <c r="B101" s="62" t="inlineStr">
         <is>
           <t>CO-14104</t>
         </is>
@@ -4178,7 +4213,7 @@
           <t>9715300</t>
         </is>
       </c>
-      <c r="B102" s="13" t="inlineStr">
+      <c r="B102" s="62" t="inlineStr">
         <is>
           <t>CO-14105</t>
         </is>
@@ -4225,7 +4260,7 @@
           <t>9715300</t>
         </is>
       </c>
-      <c r="B103" s="13" t="inlineStr">
+      <c r="B103" s="62" t="inlineStr">
         <is>
           <t>CO-14106</t>
         </is>
@@ -4272,7 +4307,7 @@
           <t>9715300</t>
         </is>
       </c>
-      <c r="B104" s="13" t="inlineStr">
+      <c r="B104" s="62" t="inlineStr">
         <is>
           <t>CO-14107</t>
         </is>
@@ -4319,7 +4354,7 @@
           <t>9722D10</t>
         </is>
       </c>
-      <c r="B105" s="13" t="inlineStr">
+      <c r="B105" s="62" t="inlineStr">
         <is>
           <t>CO-14108</t>
         </is>
@@ -4516,7 +4551,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M112" s="13" t="inlineStr">
+      <c r="M112" s="62" t="inlineStr">
         <is>
           <t>ASN0001</t>
         </is>
@@ -4652,7 +4687,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M114" s="13" t="inlineStr">
+      <c r="M114" s="62" t="inlineStr">
         <is>
           <t>ASN0002</t>
         </is>
@@ -4720,7 +4755,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M115" s="13" t="inlineStr">
+      <c r="M115" s="62" t="inlineStr">
         <is>
           <t>ASN0003</t>
         </is>
@@ -4788,7 +4823,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M116" s="13" t="inlineStr">
+      <c r="M116" s="62" t="inlineStr">
         <is>
           <t>ASN0003</t>
         </is>
@@ -4856,7 +4891,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M117" s="13" t="inlineStr">
+      <c r="M117" s="62" t="inlineStr">
         <is>
           <t>ASN0003</t>
         </is>
@@ -4924,7 +4959,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M118" s="13" t="inlineStr">
+      <c r="M118" s="62" t="inlineStr">
         <is>
           <t>ASN0003</t>
         </is>
@@ -5004,6 +5039,7 @@
       </c>
     </row>
     <row r="120" customFormat="1" s="34"/>
+    <row r="121"/>
     <row r="122">
       <c r="A122" s="39" t="inlineStr">
         <is>
@@ -5154,7 +5190,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M126" s="13" t="inlineStr">
+      <c r="M126" s="62" t="inlineStr">
         <is>
           <t>ASN0001</t>
         </is>
@@ -5290,7 +5326,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M128" s="13" t="inlineStr">
+      <c r="M128" s="62" t="inlineStr">
         <is>
           <t>ASN0002</t>
         </is>
@@ -5358,7 +5394,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M129" s="13" t="inlineStr">
+      <c r="M129" s="62" t="inlineStr">
         <is>
           <t>ASN0003</t>
         </is>
@@ -5426,7 +5462,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M130" s="13" t="inlineStr">
+      <c r="M130" s="62" t="inlineStr">
         <is>
           <t>ASN0003</t>
         </is>
@@ -5494,7 +5530,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M131" s="13" t="inlineStr">
+      <c r="M131" s="62" t="inlineStr">
         <is>
           <t>ASN0003</t>
         </is>
@@ -5630,7 +5666,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M133" s="56" t="inlineStr">
+      <c r="M133" s="63" t="inlineStr">
         <is>
           <t>ASN0003</t>
         </is>
@@ -5647,6 +5683,53 @@
     <row r="143" customFormat="1" s="34"/>
     <row r="144" customFormat="1" s="34"/>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B5" location="'Sheet1'!B13" tooltip="NSP.TB_R_H0253_ORDER_CONTROL_PRE (setelah XD08)"/>
+    <hyperlink ref="B6" location="'Sheet1'!B14" tooltip="NSP.TB_R_H0253_ORDER_CONTROL_PRE (setelah XD08)"/>
+    <hyperlink ref="M21" location="'Sheet2'!R12" tooltip="TB_R_INSTRUCTION (Sheet2)"/>
+    <hyperlink ref="B29" location="'Sheet1'!B38" tooltip="NSP.TB_R_H0253_ORDER_CONTROL_PRE (setelah XD08)"/>
+    <hyperlink ref="B30" location="'Sheet1'!B39" tooltip="NSP.TB_R_H0253_ORDER_CONTROL_PRE (setelah XD08)"/>
+    <hyperlink ref="B31" location="'Sheet1'!B40" tooltip="NSP.TB_R_H0253_ORDER_CONTROL_PRE (setelah XD08)"/>
+    <hyperlink ref="M38" location="'Sheet2'!R12" tooltip="TB_R_INSTRUCTION (Sheet2)"/>
+    <hyperlink ref="M47" location="'Sheet2'!R12" tooltip="TB_R_INSTRUCTION (Sheet2)"/>
+    <hyperlink ref="M49" location="'Sheet2'!R13" tooltip="TB_R_INSTRUCTION (Sheet2)"/>
+    <hyperlink ref="B56" location="'Sheet1'!B70" tooltip="NSP.TB_R_H0253_ORDER_CONTROL_PRE (setelah XD08)"/>
+    <hyperlink ref="B57" location="'Sheet1'!B71" tooltip="NSP.TB_R_H0253_ORDER_CONTROL_PRE (setelah XD08)"/>
+    <hyperlink ref="B58" location="'Sheet1'!B72" tooltip="NSP.TB_R_H0253_ORDER_CONTROL_PRE (setelah XD08)"/>
+    <hyperlink ref="B59" location="'Sheet1'!B76" tooltip="NSP.TB_R_H0253_ORDER_CONTROL_PRE (setelah XD08)"/>
+    <hyperlink ref="B60" location="'Sheet1'!B73" tooltip="NSP.TB_R_H0253_ORDER_CONTROL_PRE (setelah XD08)"/>
+    <hyperlink ref="B61" location="'Sheet1'!B74" tooltip="NSP.TB_R_H0253_ORDER_CONTROL_PRE (setelah XD08)"/>
+    <hyperlink ref="B62" location="'Sheet1'!B75" tooltip="NSP.TB_R_H0253_ORDER_CONTROL_PRE (setelah XD08)"/>
+    <hyperlink ref="B63" location="'Sheet1'!B77" tooltip="NSP.TB_R_H0253_ORDER_CONTROL_PRE (setelah XD08)"/>
+    <hyperlink ref="M70" location="'Sheet2'!R12" tooltip="TB_R_INSTRUCTION (Sheet2)"/>
+    <hyperlink ref="M72" location="'Sheet2'!R13" tooltip="TB_R_INSTRUCTION (Sheet2)"/>
+    <hyperlink ref="M84" location="'Sheet2'!R12" tooltip="TB_R_INSTRUCTION (Sheet2)"/>
+    <hyperlink ref="M86" location="'Sheet2'!R13" tooltip="TB_R_INSTRUCTION (Sheet2)"/>
+    <hyperlink ref="M87" location="'Sheet2'!R14" tooltip="TB_R_INSTRUCTION (Sheet2)"/>
+    <hyperlink ref="M88" location="'Sheet2'!R15" tooltip="TB_R_INSTRUCTION (Sheet2)"/>
+    <hyperlink ref="M89" location="'Sheet2'!R16" tooltip="TB_R_INSTRUCTION (Sheet2)"/>
+    <hyperlink ref="M90" location="'Sheet2'!R17" tooltip="TB_R_INSTRUCTION (Sheet2)"/>
+    <hyperlink ref="B98" location="'Sheet1'!B112" tooltip="NSP.TB_R_H0253_ORDER_CONTROL_PRE (setelah XD08)"/>
+    <hyperlink ref="B99" location="'Sheet1'!B113" tooltip="NSP.TB_R_H0253_ORDER_CONTROL_PRE (setelah XD08)"/>
+    <hyperlink ref="B100" location="'Sheet1'!B114" tooltip="NSP.TB_R_H0253_ORDER_CONTROL_PRE (setelah XD08)"/>
+    <hyperlink ref="B101" location="'Sheet1'!B118" tooltip="NSP.TB_R_H0253_ORDER_CONTROL_PRE (setelah XD08)"/>
+    <hyperlink ref="B102" location="'Sheet1'!B115" tooltip="NSP.TB_R_H0253_ORDER_CONTROL_PRE (setelah XD08)"/>
+    <hyperlink ref="B103" location="'Sheet1'!B116" tooltip="NSP.TB_R_H0253_ORDER_CONTROL_PRE (setelah XD08)"/>
+    <hyperlink ref="B104" location="'Sheet1'!B117" tooltip="NSP.TB_R_H0253_ORDER_CONTROL_PRE (setelah XD08)"/>
+    <hyperlink ref="B105" location="'Sheet1'!B119" tooltip="NSP.TB_R_H0253_ORDER_CONTROL_PRE (setelah XD08)"/>
+    <hyperlink ref="M112" location="'Sheet2'!R12" tooltip="TB_R_INSTRUCTION (Sheet2)"/>
+    <hyperlink ref="M114" location="'Sheet2'!R13" tooltip="TB_R_INSTRUCTION (Sheet2)"/>
+    <hyperlink ref="M115" location="'Sheet2'!R14" tooltip="TB_R_INSTRUCTION (Sheet2)"/>
+    <hyperlink ref="M116" location="'Sheet2'!R15" tooltip="TB_R_INSTRUCTION (Sheet2)"/>
+    <hyperlink ref="M117" location="'Sheet2'!R16" tooltip="TB_R_INSTRUCTION (Sheet2)"/>
+    <hyperlink ref="M118" location="'Sheet2'!R17" tooltip="TB_R_INSTRUCTION (Sheet2)"/>
+    <hyperlink ref="M126" location="'Sheet2'!R12" tooltip="TB_R_INSTRUCTION (Sheet2)"/>
+    <hyperlink ref="M128" location="'Sheet2'!R13" tooltip="TB_R_INSTRUCTION (Sheet2)"/>
+    <hyperlink ref="M129" location="'Sheet2'!R14" tooltip="TB_R_INSTRUCTION (Sheet2)"/>
+    <hyperlink ref="M130" location="'Sheet2'!R15" tooltip="TB_R_INSTRUCTION (Sheet2)"/>
+    <hyperlink ref="M131" location="'Sheet2'!R16" tooltip="TB_R_INSTRUCTION (Sheet2)"/>
+    <hyperlink ref="M133" location="'Sheet2'!R18" tooltip="TB_R_INSTRUCTION (Sheet2)"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait"/>
 </worksheet>
@@ -5658,7 +5741,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T23"/>
+  <dimension ref="A1:U24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="22" customWidth="1" style="26" min="2" max="2"/>
@@ -5798,7 +5881,7 @@
           <t>0001</t>
         </is>
       </c>
-      <c r="E4" s="46" t="inlineStr">
+      <c r="E4" s="64" t="inlineStr">
         <is>
           <t>T0409011</t>
         </is>
@@ -5816,7 +5899,7 @@
       <c r="H4" s="46" t="n">
         <v>6</v>
       </c>
-      <c r="I4" s="58" t="n">
+      <c r="I4" s="65" t="n">
         <v>46311</v>
       </c>
       <c r="J4" s="46" t="inlineStr">
@@ -5829,12 +5912,12 @@
           <t>16/10/2026</t>
         </is>
       </c>
-      <c r="M4" s="46" t="inlineStr">
+      <c r="M4" s="64" t="inlineStr">
         <is>
           <t>T0409011</t>
         </is>
       </c>
-      <c r="N4" s="46" t="inlineStr">
+      <c r="N4" s="64" t="inlineStr">
         <is>
           <t>3126035911</t>
         </is>
@@ -5877,7 +5960,7 @@
           <t>0001</t>
         </is>
       </c>
-      <c r="E5" s="46" t="inlineStr">
+      <c r="E5" s="64" t="inlineStr">
         <is>
           <t>T0409012</t>
         </is>
@@ -5895,7 +5978,7 @@
       <c r="H5" s="46" t="n">
         <v>6</v>
       </c>
-      <c r="I5" s="58" t="n">
+      <c r="I5" s="65" t="n">
         <v>46311</v>
       </c>
       <c r="J5" s="46" t="inlineStr">
@@ -5908,12 +5991,12 @@
           <t>17/10/2026</t>
         </is>
       </c>
-      <c r="M5" s="46" t="inlineStr">
+      <c r="M5" s="64" t="inlineStr">
         <is>
           <t>T0409012</t>
         </is>
       </c>
-      <c r="N5" s="46" t="inlineStr">
+      <c r="N5" s="64" t="inlineStr">
         <is>
           <t>3126035912</t>
         </is>
@@ -5956,7 +6039,7 @@
           <t>0001</t>
         </is>
       </c>
-      <c r="E6" s="46" t="inlineStr">
+      <c r="E6" s="64" t="inlineStr">
         <is>
           <t>T0409013</t>
         </is>
@@ -5974,7 +6057,7 @@
       <c r="H6" s="46" t="n">
         <v>6</v>
       </c>
-      <c r="I6" s="58" t="n">
+      <c r="I6" s="65" t="n">
         <v>46312</v>
       </c>
       <c r="J6" s="46" t="inlineStr">
@@ -5987,12 +6070,12 @@
           <t>18/10/2026</t>
         </is>
       </c>
-      <c r="M6" s="46" t="inlineStr">
+      <c r="M6" s="64" t="inlineStr">
         <is>
           <t>T0409013</t>
         </is>
       </c>
-      <c r="N6" s="46" t="inlineStr">
+      <c r="N6" s="64" t="inlineStr">
         <is>
           <t>3126035913</t>
         </is>
@@ -6035,7 +6118,7 @@
           <t>0001</t>
         </is>
       </c>
-      <c r="E7" s="46" t="inlineStr">
+      <c r="E7" s="64" t="inlineStr">
         <is>
           <t>T0409014</t>
         </is>
@@ -6053,7 +6136,7 @@
       <c r="H7" s="46" t="n">
         <v>12</v>
       </c>
-      <c r="I7" s="58" t="n">
+      <c r="I7" s="65" t="n">
         <v>46313</v>
       </c>
       <c r="J7" s="46" t="inlineStr">
@@ -6066,12 +6149,12 @@
           <t>18/10/2026</t>
         </is>
       </c>
-      <c r="M7" s="46" t="inlineStr">
+      <c r="M7" s="64" t="inlineStr">
         <is>
           <t>T0409014</t>
         </is>
       </c>
-      <c r="N7" s="46" t="inlineStr">
+      <c r="N7" s="64" t="inlineStr">
         <is>
           <t>3126035914</t>
         </is>
@@ -6234,12 +6317,12 @@
           <t>9715300</t>
         </is>
       </c>
-      <c r="I12" s="46" t="inlineStr">
+      <c r="I12" s="64" t="inlineStr">
         <is>
           <t>CO-14101</t>
         </is>
       </c>
-      <c r="J12" s="58" t="n">
+      <c r="J12" s="65" t="n">
         <v>46310</v>
       </c>
       <c r="K12" s="46" t="inlineStr">
@@ -6260,12 +6343,12 @@
       <c r="N12" s="46" t="n">
         <v>6</v>
       </c>
-      <c r="O12" s="46" t="inlineStr">
+      <c r="O12" s="64" t="inlineStr">
         <is>
           <t>T0409011</t>
         </is>
       </c>
-      <c r="P12" s="46" t="inlineStr">
+      <c r="P12" s="64" t="inlineStr">
         <is>
           <t>3126035911</t>
         </is>
@@ -6317,12 +6400,12 @@
           <t>9722D10</t>
         </is>
       </c>
-      <c r="I13" s="46" t="inlineStr">
+      <c r="I13" s="64" t="inlineStr">
         <is>
           <t>CO-14103</t>
         </is>
       </c>
-      <c r="J13" s="58" t="n">
+      <c r="J13" s="65" t="n">
         <v>46311</v>
       </c>
       <c r="K13" s="46" t="inlineStr">
@@ -6343,12 +6426,12 @@
       <c r="N13" s="46" t="n">
         <v>6</v>
       </c>
-      <c r="O13" s="46" t="inlineStr">
+      <c r="O13" s="64" t="inlineStr">
         <is>
           <t>T0409012</t>
         </is>
       </c>
-      <c r="P13" s="46" t="inlineStr">
+      <c r="P13" s="64" t="inlineStr">
         <is>
           <t>3126035912</t>
         </is>
@@ -6400,12 +6483,12 @@
           <t>9715300</t>
         </is>
       </c>
-      <c r="I14" s="46" t="inlineStr">
+      <c r="I14" s="64" t="inlineStr">
         <is>
           <t>CO-14105</t>
         </is>
       </c>
-      <c r="J14" s="58" t="n">
+      <c r="J14" s="65" t="n">
         <v>46312</v>
       </c>
       <c r="K14" s="46" t="inlineStr">
@@ -6426,12 +6509,12 @@
       <c r="N14" s="46" t="n">
         <v>6</v>
       </c>
-      <c r="O14" s="46" t="inlineStr">
+      <c r="O14" s="64" t="inlineStr">
         <is>
           <t>T0409013</t>
         </is>
       </c>
-      <c r="P14" s="46" t="inlineStr">
+      <c r="P14" s="64" t="inlineStr">
         <is>
           <t>3126035913</t>
         </is>
@@ -6487,12 +6570,12 @@
           <t>9715300</t>
         </is>
       </c>
-      <c r="I15" s="46" t="inlineStr">
+      <c r="I15" s="64" t="inlineStr">
         <is>
           <t>CO-14106</t>
         </is>
       </c>
-      <c r="J15" s="58" t="n">
+      <c r="J15" s="65" t="n">
         <v>46312</v>
       </c>
       <c r="K15" s="46" t="inlineStr">
@@ -6513,12 +6596,12 @@
       <c r="N15" s="46" t="n">
         <v>3</v>
       </c>
-      <c r="O15" s="46" t="inlineStr">
+      <c r="O15" s="64" t="inlineStr">
         <is>
           <t>T0409014</t>
         </is>
       </c>
-      <c r="P15" s="46" t="inlineStr">
+      <c r="P15" s="64" t="inlineStr">
         <is>
           <t>3126035914</t>
         </is>
@@ -6570,12 +6653,12 @@
           <t>9715300</t>
         </is>
       </c>
-      <c r="I16" s="46" t="inlineStr">
+      <c r="I16" s="64" t="inlineStr">
         <is>
           <t>CO-14107</t>
         </is>
       </c>
-      <c r="J16" s="58" t="n">
+      <c r="J16" s="65" t="n">
         <v>46312</v>
       </c>
       <c r="K16" s="46" t="inlineStr">
@@ -6596,12 +6679,12 @@
       <c r="N16" s="46" t="n">
         <v>3</v>
       </c>
-      <c r="O16" s="46" t="inlineStr">
+      <c r="O16" s="64" t="inlineStr">
         <is>
           <t>T0409014</t>
         </is>
       </c>
-      <c r="P16" s="46" t="inlineStr">
+      <c r="P16" s="64" t="inlineStr">
         <is>
           <t>3126035914</t>
         </is>
@@ -6657,12 +6740,12 @@
           <t>9722D10</t>
         </is>
       </c>
-      <c r="I17" s="46" t="inlineStr">
+      <c r="I17" s="64" t="inlineStr">
         <is>
           <t>CO-14104</t>
         </is>
       </c>
-      <c r="J17" s="58" t="n">
+      <c r="J17" s="65" t="n">
         <v>46312</v>
       </c>
       <c r="K17" s="46" t="inlineStr">
@@ -6683,12 +6766,12 @@
       <c r="N17" s="46" t="n">
         <v>6</v>
       </c>
-      <c r="O17" s="46" t="inlineStr">
+      <c r="O17" s="64" t="inlineStr">
         <is>
           <t>T0409014</t>
         </is>
       </c>
-      <c r="P17" s="46" t="inlineStr">
+      <c r="P17" s="64" t="inlineStr">
         <is>
           <t>3126035914</t>
         </is>
@@ -6744,12 +6827,12 @@
           <t>9722D10</t>
         </is>
       </c>
-      <c r="I18" s="59" t="inlineStr">
+      <c r="I18" s="66" t="inlineStr">
         <is>
           <t>CO-14108</t>
         </is>
       </c>
-      <c r="J18" s="60" t="n">
+      <c r="J18" s="67" t="n">
         <v>46313</v>
       </c>
       <c r="K18" s="46" t="inlineStr">
@@ -6770,12 +6853,12 @@
       <c r="N18" s="46" t="n">
         <v>6</v>
       </c>
-      <c r="O18" s="46" t="inlineStr">
+      <c r="O18" s="64" t="inlineStr">
         <is>
           <t>T0409014</t>
         </is>
       </c>
-      <c r="P18" s="46" t="inlineStr">
+      <c r="P18" s="64" t="inlineStr">
         <is>
           <t>3126035914</t>
         </is>
@@ -6886,7 +6969,7 @@
       <c r="C23" s="46" t="n">
         <v>1</v>
       </c>
-      <c r="D23" s="46" t="inlineStr">
+      <c r="D23" s="64" t="inlineStr">
         <is>
           <t>ASN0003</t>
         </is>
@@ -6901,7 +6984,7 @@
           <t>PART-X</t>
         </is>
       </c>
-      <c r="G23" s="46" t="inlineStr">
+      <c r="G23" s="64" t="inlineStr">
         <is>
           <t>CO-14104</t>
         </is>
@@ -6911,7 +6994,7 @@
           <t>0000001</t>
         </is>
       </c>
-      <c r="I23" s="46" t="inlineStr">
+      <c r="I23" s="64" t="inlineStr">
         <is>
           <t>CO-14108</t>
         </is>
@@ -6924,10 +7007,10 @@
       <c r="K23" s="46" t="n">
         <v>6</v>
       </c>
-      <c r="L23" s="46" t="n">
-        <v>6</v>
-      </c>
-      <c r="M23" s="46" t="n">
+      <c r="L23" s="64" t="n">
+        <v>6</v>
+      </c>
+      <c r="M23" s="64" t="n">
         <v>6</v>
       </c>
       <c r="N23" s="46" t="inlineStr">
@@ -6936,7 +7019,48 @@
         </is>
       </c>
     </row>
+    <row r="24"/>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="E4" location="'Sheet2'!M4" tooltip="TB_R_PRA_DAILY_ORDER_MAPPED"/>
+    <hyperlink ref="M4" location="'Sheet2'!E4" tooltip="TB_R_PRA_DAILY_ORDER_PART"/>
+    <hyperlink ref="N4" location="'Sheet2'!C4" tooltip="TB_R_PRA_DAILY_ORDER_PART"/>
+    <hyperlink ref="E5" location="'Sheet2'!M5" tooltip="TB_R_PRA_DAILY_ORDER_MAPPED"/>
+    <hyperlink ref="M5" location="'Sheet2'!E5" tooltip="TB_R_PRA_DAILY_ORDER_PART"/>
+    <hyperlink ref="N5" location="'Sheet2'!C5" tooltip="TB_R_PRA_DAILY_ORDER_PART"/>
+    <hyperlink ref="E6" location="'Sheet2'!M6" tooltip="TB_R_PRA_DAILY_ORDER_MAPPED"/>
+    <hyperlink ref="M6" location="'Sheet2'!E6" tooltip="TB_R_PRA_DAILY_ORDER_PART"/>
+    <hyperlink ref="N6" location="'Sheet2'!C6" tooltip="TB_R_PRA_DAILY_ORDER_PART"/>
+    <hyperlink ref="E7" location="'Sheet2'!M7" tooltip="TB_R_PRA_DAILY_ORDER_MAPPED"/>
+    <hyperlink ref="M7" location="'Sheet2'!E7" tooltip="TB_R_PRA_DAILY_ORDER_PART"/>
+    <hyperlink ref="N7" location="'Sheet2'!C7" tooltip="TB_R_PRA_DAILY_ORDER_PART"/>
+    <hyperlink ref="I12" location="'Sheet1'!B21" tooltip="NSP.TB_R_H0253_ORDER_CONTROL_PRE (Sheet1)"/>
+    <hyperlink ref="O12" location="'Sheet2'!E4" tooltip="TB_R_PRA_DAILY_ORDER_PART"/>
+    <hyperlink ref="P12" location="'Sheet2'!C4" tooltip="TB_R_PRA_DAILY_ORDER_PART"/>
+    <hyperlink ref="I13" location="'Sheet1'!B49" tooltip="NSP.TB_R_H0253_ORDER_CONTROL_PRE (Sheet1)"/>
+    <hyperlink ref="O13" location="'Sheet2'!E5" tooltip="TB_R_PRA_DAILY_ORDER_PART"/>
+    <hyperlink ref="P13" location="'Sheet2'!C5" tooltip="TB_R_PRA_DAILY_ORDER_PART"/>
+    <hyperlink ref="I14" location="'Sheet1'!B87" tooltip="NSP.TB_R_H0253_ORDER_CONTROL_PRE (Sheet1)"/>
+    <hyperlink ref="O14" location="'Sheet2'!E6" tooltip="TB_R_PRA_DAILY_ORDER_PART"/>
+    <hyperlink ref="P14" location="'Sheet2'!C6" tooltip="TB_R_PRA_DAILY_ORDER_PART"/>
+    <hyperlink ref="I15" location="'Sheet1'!B88" tooltip="NSP.TB_R_H0253_ORDER_CONTROL_PRE (Sheet1)"/>
+    <hyperlink ref="O15" location="'Sheet2'!E7" tooltip="TB_R_PRA_DAILY_ORDER_PART"/>
+    <hyperlink ref="P15" location="'Sheet2'!C7" tooltip="TB_R_PRA_DAILY_ORDER_PART"/>
+    <hyperlink ref="I16" location="'Sheet1'!B89" tooltip="NSP.TB_R_H0253_ORDER_CONTROL_PRE (Sheet1)"/>
+    <hyperlink ref="O16" location="'Sheet2'!E7" tooltip="TB_R_PRA_DAILY_ORDER_PART"/>
+    <hyperlink ref="P16" location="'Sheet2'!C7" tooltip="TB_R_PRA_DAILY_ORDER_PART"/>
+    <hyperlink ref="I17" location="'Sheet1'!B90" tooltip="NSP.TB_R_H0253_ORDER_CONTROL_PRE (Sheet1)"/>
+    <hyperlink ref="O17" location="'Sheet2'!E7" tooltip="TB_R_PRA_DAILY_ORDER_PART"/>
+    <hyperlink ref="P17" location="'Sheet2'!C7" tooltip="TB_R_PRA_DAILY_ORDER_PART"/>
+    <hyperlink ref="I18" location="'Sheet1'!B133" tooltip="NSP.TB_R_H0253_ORDER_CONTROL_PRE (Sheet1)"/>
+    <hyperlink ref="O18" location="'Sheet2'!E7" tooltip="TB_R_PRA_DAILY_ORDER_PART"/>
+    <hyperlink ref="P18" location="'Sheet2'!C7" tooltip="TB_R_PRA_DAILY_ORDER_PART"/>
+    <hyperlink ref="D23" location="'Sheet2'!R18" tooltip="TB_R_INSTRUCTION"/>
+    <hyperlink ref="G23" location="'Sheet1'!B132" tooltip="NSP.TB_R_H0253_ORDER_CONTROL_PRE (Sheet1)"/>
+    <hyperlink ref="I23" location="'Sheet1'!B133" tooltip="NSP.TB_R_H0253_ORDER_CONTROL_PRE (Sheet1)"/>
+    <hyperlink ref="L23" location="'Sheet2'!C17" tooltip="TB_R_INSTRUCTION (before)"/>
+    <hyperlink ref="M23" location="'Sheet2'!C18" tooltip="TB_R_INSTRUCTION (after)"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -6976,7 +7100,13 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
+    <row r="2">
+      <c r="A2" s="68" t="inlineStr">
+        <is>
+          <t>Teks biru bergaris bawah = hyperlink ke tabel terkait (PO_NO / MANIFEST_NO → TB_R_PRA_DAILY_ORDER_PART, CUSTOMER_ORDER_NO → H0253 replicate di Sheet1).</t>
+        </is>
+      </c>
+    </row>
     <row r="3">
       <c r="A3" s="57" t="inlineStr">
         <is>
@@ -7080,7 +7210,7 @@
           <t>PART-X</t>
         </is>
       </c>
-      <c r="C5" s="58" t="n">
+      <c r="C5" s="65" t="n">
         <v>46310</v>
       </c>
       <c r="D5" s="46" t="inlineStr">
@@ -7088,7 +7218,7 @@
           <t>9715300</t>
         </is>
       </c>
-      <c r="E5" s="46" t="inlineStr">
+      <c r="E5" s="64" t="inlineStr">
         <is>
           <t>CO-14101</t>
         </is>
@@ -7104,12 +7234,12 @@
       <c r="H5" s="46" t="n">
         <v>6</v>
       </c>
-      <c r="I5" s="46" t="inlineStr">
+      <c r="I5" s="64" t="inlineStr">
         <is>
           <t>T0409011</t>
         </is>
       </c>
-      <c r="J5" s="46" t="inlineStr">
+      <c r="J5" s="64" t="inlineStr">
         <is>
           <t>3126035911</t>
         </is>
@@ -7246,7 +7376,7 @@
           <t>PART-X</t>
         </is>
       </c>
-      <c r="C9" s="58" t="n">
+      <c r="C9" s="65" t="n">
         <v>46311</v>
       </c>
       <c r="D9" s="46" t="inlineStr">
@@ -7254,7 +7384,7 @@
           <t>9722D10</t>
         </is>
       </c>
-      <c r="E9" s="46" t="inlineStr">
+      <c r="E9" s="64" t="inlineStr">
         <is>
           <t>CO-14103</t>
         </is>
@@ -7270,12 +7400,12 @@
       <c r="H9" s="46" t="n">
         <v>6</v>
       </c>
-      <c r="I9" s="46" t="inlineStr">
+      <c r="I9" s="64" t="inlineStr">
         <is>
           <t>T0409012</t>
         </is>
       </c>
-      <c r="J9" s="46" t="inlineStr">
+      <c r="J9" s="64" t="inlineStr">
         <is>
           <t>3126035912</t>
         </is>
@@ -7412,7 +7542,7 @@
           <t>PART-X</t>
         </is>
       </c>
-      <c r="C13" s="58" t="n">
+      <c r="C13" s="65" t="n">
         <v>46312</v>
       </c>
       <c r="D13" s="46" t="inlineStr">
@@ -7420,7 +7550,7 @@
           <t>9715300</t>
         </is>
       </c>
-      <c r="E13" s="46" t="inlineStr">
+      <c r="E13" s="64" t="inlineStr">
         <is>
           <t>CO-14105</t>
         </is>
@@ -7436,12 +7566,12 @@
       <c r="H13" s="46" t="n">
         <v>6</v>
       </c>
-      <c r="I13" s="46" t="inlineStr">
+      <c r="I13" s="64" t="inlineStr">
         <is>
           <t>T0409013</t>
         </is>
       </c>
-      <c r="J13" s="46" t="inlineStr">
+      <c r="J13" s="64" t="inlineStr">
         <is>
           <t>3126035913</t>
         </is>
@@ -7483,7 +7613,7 @@
           <t>PART-X</t>
         </is>
       </c>
-      <c r="C14" s="58" t="n">
+      <c r="C14" s="65" t="n">
         <v>46312</v>
       </c>
       <c r="D14" s="46" t="inlineStr">
@@ -7491,7 +7621,7 @@
           <t>9715300</t>
         </is>
       </c>
-      <c r="E14" s="46" t="inlineStr">
+      <c r="E14" s="64" t="inlineStr">
         <is>
           <t>CO-14106</t>
         </is>
@@ -7507,12 +7637,12 @@
       <c r="H14" s="46" t="n">
         <v>3</v>
       </c>
-      <c r="I14" s="46" t="inlineStr">
+      <c r="I14" s="64" t="inlineStr">
         <is>
           <t>T0409014</t>
         </is>
       </c>
-      <c r="J14" s="46" t="inlineStr">
+      <c r="J14" s="64" t="inlineStr">
         <is>
           <t>3126035914</t>
         </is>
@@ -7550,7 +7680,7 @@
           <t>PART-X</t>
         </is>
       </c>
-      <c r="C15" s="58" t="n">
+      <c r="C15" s="65" t="n">
         <v>46312</v>
       </c>
       <c r="D15" s="46" t="inlineStr">
@@ -7558,7 +7688,7 @@
           <t>9715300</t>
         </is>
       </c>
-      <c r="E15" s="46" t="inlineStr">
+      <c r="E15" s="64" t="inlineStr">
         <is>
           <t>CO-14107</t>
         </is>
@@ -7574,12 +7704,12 @@
       <c r="H15" s="46" t="n">
         <v>3</v>
       </c>
-      <c r="I15" s="46" t="inlineStr">
+      <c r="I15" s="64" t="inlineStr">
         <is>
           <t>T0409014</t>
         </is>
       </c>
-      <c r="J15" s="46" t="inlineStr">
+      <c r="J15" s="64" t="inlineStr">
         <is>
           <t>3126035914</t>
         </is>
@@ -7617,7 +7747,7 @@
           <t>PART-X</t>
         </is>
       </c>
-      <c r="C16" s="58" t="n">
+      <c r="C16" s="65" t="n">
         <v>46312</v>
       </c>
       <c r="D16" s="46" t="inlineStr">
@@ -7625,7 +7755,7 @@
           <t>9722D10</t>
         </is>
       </c>
-      <c r="E16" s="46" t="inlineStr">
+      <c r="E16" s="64" t="inlineStr">
         <is>
           <t>CO-14104</t>
         </is>
@@ -7641,12 +7771,12 @@
       <c r="H16" s="46" t="n">
         <v>6</v>
       </c>
-      <c r="I16" s="46" t="inlineStr">
+      <c r="I16" s="64" t="inlineStr">
         <is>
           <t>T0409014</t>
         </is>
       </c>
-      <c r="J16" s="46" t="inlineStr">
+      <c r="J16" s="64" t="inlineStr">
         <is>
           <t>3126035914</t>
         </is>
@@ -7684,7 +7814,7 @@
           <t>PART-X</t>
         </is>
       </c>
-      <c r="C17" s="58" t="n">
+      <c r="C17" s="65" t="n">
         <v>46313</v>
       </c>
       <c r="D17" s="46" t="inlineStr">
@@ -7692,7 +7822,7 @@
           <t>9722D10</t>
         </is>
       </c>
-      <c r="E17" s="46" t="inlineStr">
+      <c r="E17" s="64" t="inlineStr">
         <is>
           <t>CO-14108</t>
         </is>
@@ -7747,6 +7877,27 @@
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="E5" location="'Sheet1'!B13" tooltip="NSP.TB_R_H0253_ORDER_CONTROL_PRE (Sheet1)"/>
+    <hyperlink ref="I5" location="'Sheet2'!E4" tooltip="TB_R_PRA_DAILY_ORDER_PART (Sheet2)"/>
+    <hyperlink ref="J5" location="'Sheet2'!C4" tooltip="TB_R_PRA_DAILY_ORDER_PART (Sheet2)"/>
+    <hyperlink ref="E9" location="'Sheet1'!B40" tooltip="NSP.TB_R_H0253_ORDER_CONTROL_PRE (Sheet1)"/>
+    <hyperlink ref="I9" location="'Sheet2'!E5" tooltip="TB_R_PRA_DAILY_ORDER_PART (Sheet2)"/>
+    <hyperlink ref="J9" location="'Sheet2'!C5" tooltip="TB_R_PRA_DAILY_ORDER_PART (Sheet2)"/>
+    <hyperlink ref="E13" location="'Sheet1'!B73" tooltip="NSP.TB_R_H0253_ORDER_CONTROL_PRE (Sheet1)"/>
+    <hyperlink ref="I13" location="'Sheet2'!E6" tooltip="TB_R_PRA_DAILY_ORDER_PART (Sheet2)"/>
+    <hyperlink ref="J13" location="'Sheet2'!C6" tooltip="TB_R_PRA_DAILY_ORDER_PART (Sheet2)"/>
+    <hyperlink ref="E14" location="'Sheet1'!B74" tooltip="NSP.TB_R_H0253_ORDER_CONTROL_PRE (Sheet1)"/>
+    <hyperlink ref="I14" location="'Sheet2'!E7" tooltip="TB_R_PRA_DAILY_ORDER_PART (Sheet2)"/>
+    <hyperlink ref="J14" location="'Sheet2'!C7" tooltip="TB_R_PRA_DAILY_ORDER_PART (Sheet2)"/>
+    <hyperlink ref="E15" location="'Sheet1'!B75" tooltip="NSP.TB_R_H0253_ORDER_CONTROL_PRE (Sheet1)"/>
+    <hyperlink ref="I15" location="'Sheet2'!E7" tooltip="TB_R_PRA_DAILY_ORDER_PART (Sheet2)"/>
+    <hyperlink ref="J15" location="'Sheet2'!C7" tooltip="TB_R_PRA_DAILY_ORDER_PART (Sheet2)"/>
+    <hyperlink ref="E16" location="'Sheet1'!B76" tooltip="NSP.TB_R_H0253_ORDER_CONTROL_PRE (Sheet1)"/>
+    <hyperlink ref="I16" location="'Sheet2'!E7" tooltip="TB_R_PRA_DAILY_ORDER_PART (Sheet2)"/>
+    <hyperlink ref="J16" location="'Sheet2'!C7" tooltip="TB_R_PRA_DAILY_ORDER_PART (Sheet2)"/>
+    <hyperlink ref="E17" location="'Sheet1'!B77" tooltip="NSP.TB_R_H0253_ORDER_CONTROL_PRE (Sheet1)"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Web uses the simulasi_asn_rev data: ASN Simulation page, scenario 5 with CO-14115
- deliverables/simulasi_asn: generator of simulasi_asn_rev.xlsx (template, sim_build,
  add_links) and export_web.py → app/src/features/asnSim/simData.ts; build.sh runs all.
- New menu ASN > ASN Simulation: the workbook day by day (G-System, NSP replicate, XD09
  Search) and the NSP tables, same values and highlights.
- Cancel Order Simulation scenario 5 uses CO-14115 (ASN0006 / ASN0007, 20-22 Oct).
- Template highlight of ORDER_STATUS no longer copied to every row.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QL8Do8Pd2rXEDNa1ifG2RK
</commit_message>
<xml_diff>
--- a/deliverables/simulasi_asn_rev.xlsx
+++ b/deliverables/simulasi_asn_rev.xlsx
@@ -218,7 +218,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="71">
+  <cellXfs count="72">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -359,6 +359,9 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -842,7 +845,7 @@
           <t>9715300</t>
         </is>
       </c>
-      <c r="B5" s="63" t="inlineStr">
+      <c r="B5" s="64" t="inlineStr">
         <is>
           <t>CO-14101</t>
         </is>
@@ -889,7 +892,7 @@
           <t>9722D10</t>
         </is>
       </c>
-      <c r="B6" s="63" t="inlineStr">
+      <c r="B6" s="64" t="inlineStr">
         <is>
           <t>CO-14102</t>
         </is>
@@ -1285,7 +1288,7 @@
       <c r="H21" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I21" s="11" t="inlineStr">
+      <c r="I21" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -1305,7 +1308,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M21" s="64" t="inlineStr">
+      <c r="M21" s="65" t="inlineStr">
         <is>
           <t>ASN0001</t>
         </is>
@@ -1353,7 +1356,7 @@
       <c r="H22" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I22" s="11" t="inlineStr">
+      <c r="I22" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -1469,7 +1472,7 @@
           <t>9715300</t>
         </is>
       </c>
-      <c r="B29" s="63" t="inlineStr">
+      <c r="B29" s="64" t="inlineStr">
         <is>
           <t>CO-14101</t>
         </is>
@@ -1516,7 +1519,7 @@
           <t>9722D10</t>
         </is>
       </c>
-      <c r="B30" s="63" t="inlineStr">
+      <c r="B30" s="64" t="inlineStr">
         <is>
           <t>CO-14102</t>
         </is>
@@ -1563,7 +1566,7 @@
           <t>9722D10</t>
         </is>
       </c>
-      <c r="B31" s="63" t="inlineStr">
+      <c r="B31" s="64" t="inlineStr">
         <is>
           <t>CO-14103</t>
         </is>
@@ -1736,7 +1739,7 @@
       <c r="H38" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I38" s="11" t="inlineStr">
+      <c r="I38" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -1756,7 +1759,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M38" s="63" t="inlineStr">
+      <c r="M38" s="64" t="inlineStr">
         <is>
           <t>ASN0001</t>
         </is>
@@ -1804,7 +1807,7 @@
       <c r="H39" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I39" s="11" t="inlineStr">
+      <c r="I39" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -2035,7 +2038,7 @@
       <c r="H47" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I47" s="11" t="inlineStr">
+      <c r="I47" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -2055,7 +2058,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M47" s="63" t="inlineStr">
+      <c r="M47" s="64" t="inlineStr">
         <is>
           <t>ASN0001</t>
         </is>
@@ -2103,7 +2106,7 @@
       <c r="H48" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I48" s="11" t="inlineStr">
+      <c r="I48" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -2171,7 +2174,7 @@
       <c r="H49" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I49" s="11" t="inlineStr">
+      <c r="I49" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -2191,7 +2194,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M49" s="64" t="inlineStr">
+      <c r="M49" s="65" t="inlineStr">
         <is>
           <t>ASN0002</t>
         </is>
@@ -2287,7 +2290,7 @@
           <t>9715300</t>
         </is>
       </c>
-      <c r="B56" s="63" t="inlineStr">
+      <c r="B56" s="64" t="inlineStr">
         <is>
           <t>CO-14101</t>
         </is>
@@ -2318,7 +2321,7 @@
       <c r="H56" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I56" s="11" t="inlineStr">
+      <c r="I56" s="56" t="inlineStr">
         <is>
           <t>6</t>
         </is>
@@ -2334,7 +2337,7 @@
           <t>9722D10</t>
         </is>
       </c>
-      <c r="B57" s="63" t="inlineStr">
+      <c r="B57" s="64" t="inlineStr">
         <is>
           <t>CO-14102</t>
         </is>
@@ -2365,7 +2368,7 @@
       <c r="H57" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I57" s="11" t="inlineStr">
+      <c r="I57" s="56" t="inlineStr">
         <is>
           <t>2</t>
         </is>
@@ -2381,7 +2384,7 @@
           <t>9722D10</t>
         </is>
       </c>
-      <c r="B58" s="63" t="inlineStr">
+      <c r="B58" s="64" t="inlineStr">
         <is>
           <t>CO-14103</t>
         </is>
@@ -2428,7 +2431,7 @@
           <t>9722D10</t>
         </is>
       </c>
-      <c r="B59" s="63" t="inlineStr">
+      <c r="B59" s="64" t="inlineStr">
         <is>
           <t>CO-14104</t>
         </is>
@@ -2475,7 +2478,7 @@
           <t>9715300</t>
         </is>
       </c>
-      <c r="B60" s="63" t="inlineStr">
+      <c r="B60" s="64" t="inlineStr">
         <is>
           <t>CO-14105</t>
         </is>
@@ -2522,7 +2525,7 @@
           <t>9715300</t>
         </is>
       </c>
-      <c r="B61" s="63" t="inlineStr">
+      <c r="B61" s="64" t="inlineStr">
         <is>
           <t>CO-14106</t>
         </is>
@@ -2569,7 +2572,7 @@
           <t>9715300</t>
         </is>
       </c>
-      <c r="B62" s="63" t="inlineStr">
+      <c r="B62" s="64" t="inlineStr">
         <is>
           <t>CO-14107</t>
         </is>
@@ -2616,7 +2619,7 @@
           <t>9811100</t>
         </is>
       </c>
-      <c r="B63" s="63" t="inlineStr">
+      <c r="B63" s="64" t="inlineStr">
         <is>
           <t>CO-14109</t>
         </is>
@@ -2663,7 +2666,7 @@
           <t>982200</t>
         </is>
       </c>
-      <c r="B64" s="63" t="inlineStr">
+      <c r="B64" s="64" t="inlineStr">
         <is>
           <t>CO-14110</t>
         </is>
@@ -2836,7 +2839,7 @@
       <c r="H71" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I71" s="11" t="inlineStr">
+      <c r="I71" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -2856,7 +2859,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M71" s="63" t="inlineStr">
+      <c r="M71" s="64" t="inlineStr">
         <is>
           <t>ASN0001</t>
         </is>
@@ -2904,7 +2907,7 @@
       <c r="H72" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I72" s="11" t="inlineStr">
+      <c r="I72" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -2972,7 +2975,7 @@
       <c r="H73" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I73" s="11" t="inlineStr">
+      <c r="I73" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -2992,7 +2995,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M73" s="63" t="inlineStr">
+      <c r="M73" s="64" t="inlineStr">
         <is>
           <t>ASN0002</t>
         </is>
@@ -3543,7 +3546,7 @@
       <c r="H86" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I86" s="11" t="inlineStr">
+      <c r="I86" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -3563,7 +3566,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M86" s="63" t="inlineStr">
+      <c r="M86" s="64" t="inlineStr">
         <is>
           <t>ASN0001</t>
         </is>
@@ -3611,7 +3614,7 @@
       <c r="H87" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I87" s="11" t="inlineStr">
+      <c r="I87" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -3679,7 +3682,7 @@
       <c r="H88" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I88" s="11" t="inlineStr">
+      <c r="I88" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -3699,7 +3702,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M88" s="63" t="inlineStr">
+      <c r="M88" s="64" t="inlineStr">
         <is>
           <t>ASN0002</t>
         </is>
@@ -3747,7 +3750,7 @@
       <c r="H89" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I89" s="11" t="inlineStr">
+      <c r="I89" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -3767,7 +3770,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M89" s="64" t="inlineStr">
+      <c r="M89" s="65" t="inlineStr">
         <is>
           <t>ASN0003</t>
         </is>
@@ -3815,7 +3818,7 @@
       <c r="H90" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="I90" s="11" t="inlineStr">
+      <c r="I90" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -3835,7 +3838,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M90" s="64" t="inlineStr">
+      <c r="M90" s="65" t="inlineStr">
         <is>
           <t>ASN0003</t>
         </is>
@@ -3883,7 +3886,7 @@
       <c r="H91" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="I91" s="11" t="inlineStr">
+      <c r="I91" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -3903,7 +3906,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M91" s="64" t="inlineStr">
+      <c r="M91" s="65" t="inlineStr">
         <is>
           <t>ASN0003</t>
         </is>
@@ -3951,7 +3954,7 @@
       <c r="H92" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I92" s="11" t="inlineStr">
+      <c r="I92" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -3971,7 +3974,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M92" s="64" t="inlineStr">
+      <c r="M92" s="65" t="inlineStr">
         <is>
           <t>ASN0003</t>
         </is>
@@ -4019,7 +4022,7 @@
       <c r="H93" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I93" s="11" t="inlineStr">
+      <c r="I93" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -4039,7 +4042,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M93" s="64" t="inlineStr">
+      <c r="M93" s="65" t="inlineStr">
         <is>
           <t>ASN0003</t>
         </is>
@@ -4087,7 +4090,7 @@
       <c r="H94" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I94" s="11" t="inlineStr">
+      <c r="I94" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -4203,7 +4206,7 @@
           <t>9715300</t>
         </is>
       </c>
-      <c r="B101" s="63" t="inlineStr">
+      <c r="B101" s="64" t="inlineStr">
         <is>
           <t>CO-14101</t>
         </is>
@@ -4234,7 +4237,7 @@
       <c r="H101" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I101" s="11" t="inlineStr">
+      <c r="I101" s="56" t="inlineStr">
         <is>
           <t>6</t>
         </is>
@@ -4250,7 +4253,7 @@
           <t>9722D10</t>
         </is>
       </c>
-      <c r="B102" s="63" t="inlineStr">
+      <c r="B102" s="64" t="inlineStr">
         <is>
           <t>CO-14102</t>
         </is>
@@ -4281,7 +4284,7 @@
       <c r="H102" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I102" s="11" t="inlineStr">
+      <c r="I102" s="56" t="inlineStr">
         <is>
           <t>2</t>
         </is>
@@ -4297,7 +4300,7 @@
           <t>9722D10</t>
         </is>
       </c>
-      <c r="B103" s="63" t="inlineStr">
+      <c r="B103" s="64" t="inlineStr">
         <is>
           <t>CO-14103</t>
         </is>
@@ -4328,7 +4331,7 @@
       <c r="H103" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I103" s="11" t="inlineStr">
+      <c r="I103" s="56" t="inlineStr">
         <is>
           <t>6</t>
         </is>
@@ -4344,7 +4347,7 @@
           <t>9722D10</t>
         </is>
       </c>
-      <c r="B104" s="63" t="inlineStr">
+      <c r="B104" s="64" t="inlineStr">
         <is>
           <t>CO-14104</t>
         </is>
@@ -4395,7 +4398,7 @@
           <t>9715300</t>
         </is>
       </c>
-      <c r="B105" s="63" t="inlineStr">
+      <c r="B105" s="64" t="inlineStr">
         <is>
           <t>CO-14105</t>
         </is>
@@ -4442,7 +4445,7 @@
           <t>9715300</t>
         </is>
       </c>
-      <c r="B106" s="63" t="inlineStr">
+      <c r="B106" s="64" t="inlineStr">
         <is>
           <t>CO-14106</t>
         </is>
@@ -4489,7 +4492,7 @@
           <t>9715300</t>
         </is>
       </c>
-      <c r="B107" s="63" t="inlineStr">
+      <c r="B107" s="64" t="inlineStr">
         <is>
           <t>CO-14107</t>
         </is>
@@ -4536,7 +4539,7 @@
           <t>9811100</t>
         </is>
       </c>
-      <c r="B108" s="63" t="inlineStr">
+      <c r="B108" s="64" t="inlineStr">
         <is>
           <t>CO-14109</t>
         </is>
@@ -4583,7 +4586,7 @@
           <t>982200</t>
         </is>
       </c>
-      <c r="B109" s="63" t="inlineStr">
+      <c r="B109" s="64" t="inlineStr">
         <is>
           <t>CO-14110</t>
         </is>
@@ -4614,7 +4617,7 @@
       <c r="H109" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I109" s="11" t="inlineStr">
+      <c r="I109" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -4630,7 +4633,7 @@
           <t>9715300</t>
         </is>
       </c>
-      <c r="B110" s="63" t="inlineStr">
+      <c r="B110" s="64" t="inlineStr">
         <is>
           <t>CO-14112</t>
         </is>
@@ -4681,7 +4684,7 @@
           <t>9811100</t>
         </is>
       </c>
-      <c r="B111" s="63" t="inlineStr">
+      <c r="B111" s="64" t="inlineStr">
         <is>
           <t>CO-14113</t>
         </is>
@@ -4732,7 +4735,7 @@
           <t>982200</t>
         </is>
       </c>
-      <c r="B112" s="63" t="inlineStr">
+      <c r="B112" s="64" t="inlineStr">
         <is>
           <t>CO-14114</t>
         </is>
@@ -4909,7 +4912,7 @@
       <c r="H119" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I119" s="11" t="inlineStr">
+      <c r="I119" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -4929,7 +4932,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M119" s="63" t="inlineStr">
+      <c r="M119" s="64" t="inlineStr">
         <is>
           <t>ASN0001</t>
         </is>
@@ -4977,7 +4980,7 @@
       <c r="H120" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I120" s="11" t="inlineStr">
+      <c r="I120" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -5045,7 +5048,7 @@
       <c r="H121" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I121" s="11" t="inlineStr">
+      <c r="I121" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -5065,7 +5068,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M121" s="63" t="inlineStr">
+      <c r="M121" s="64" t="inlineStr">
         <is>
           <t>ASN0002</t>
         </is>
@@ -5113,7 +5116,7 @@
       <c r="H122" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I122" s="11" t="inlineStr">
+      <c r="I122" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -5133,7 +5136,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M122" s="63" t="inlineStr">
+      <c r="M122" s="64" t="inlineStr">
         <is>
           <t>ASN0003</t>
         </is>
@@ -5181,7 +5184,7 @@
       <c r="H123" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="I123" s="11" t="inlineStr">
+      <c r="I123" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -5201,7 +5204,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M123" s="63" t="inlineStr">
+      <c r="M123" s="64" t="inlineStr">
         <is>
           <t>ASN0003</t>
         </is>
@@ -5249,7 +5252,7 @@
       <c r="H124" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="I124" s="11" t="inlineStr">
+      <c r="I124" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -5269,7 +5272,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M124" s="63" t="inlineStr">
+      <c r="M124" s="64" t="inlineStr">
         <is>
           <t>ASN0003</t>
         </is>
@@ -5317,7 +5320,7 @@
       <c r="H125" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I125" s="11" t="inlineStr">
+      <c r="I125" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -5337,7 +5340,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M125" s="63" t="inlineStr">
+      <c r="M125" s="64" t="inlineStr">
         <is>
           <t>ASN0003</t>
         </is>
@@ -5385,7 +5388,7 @@
       <c r="H126" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I126" s="11" t="inlineStr">
+      <c r="I126" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -5405,7 +5408,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M126" s="63" t="inlineStr">
+      <c r="M126" s="64" t="inlineStr">
         <is>
           <t>ASN0003</t>
         </is>
@@ -5453,7 +5456,7 @@
       <c r="H127" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I127" s="11" t="inlineStr">
+      <c r="I127" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -5820,7 +5823,7 @@
       <c r="H137" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I137" s="11" t="inlineStr">
+      <c r="I137" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -5840,7 +5843,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M137" s="63" t="inlineStr">
+      <c r="M137" s="64" t="inlineStr">
         <is>
           <t>ASN0001</t>
         </is>
@@ -5888,7 +5891,7 @@
       <c r="H138" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I138" s="11" t="inlineStr">
+      <c r="I138" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -5956,7 +5959,7 @@
       <c r="H139" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I139" s="11" t="inlineStr">
+      <c r="I139" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -5976,7 +5979,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M139" s="63" t="inlineStr">
+      <c r="M139" s="64" t="inlineStr">
         <is>
           <t>ASN0002</t>
         </is>
@@ -6024,7 +6027,7 @@
       <c r="H140" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I140" s="11" t="inlineStr">
+      <c r="I140" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -6044,7 +6047,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M140" s="63" t="inlineStr">
+      <c r="M140" s="64" t="inlineStr">
         <is>
           <t>ASN0003</t>
         </is>
@@ -6092,7 +6095,7 @@
       <c r="H141" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="I141" s="11" t="inlineStr">
+      <c r="I141" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -6112,7 +6115,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M141" s="63" t="inlineStr">
+      <c r="M141" s="64" t="inlineStr">
         <is>
           <t>ASN0003</t>
         </is>
@@ -6160,7 +6163,7 @@
       <c r="H142" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="I142" s="11" t="inlineStr">
+      <c r="I142" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -6180,7 +6183,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M142" s="63" t="inlineStr">
+      <c r="M142" s="64" t="inlineStr">
         <is>
           <t>ASN0003</t>
         </is>
@@ -6228,7 +6231,7 @@
       <c r="H143" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I143" s="11" t="inlineStr">
+      <c r="I143" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -6248,7 +6251,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M143" s="63" t="inlineStr">
+      <c r="M143" s="64" t="inlineStr">
         <is>
           <t>ASN0003</t>
         </is>
@@ -6296,7 +6299,7 @@
       <c r="H144" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I144" s="11" t="inlineStr">
+      <c r="I144" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -6316,7 +6319,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M144" s="63" t="inlineStr">
+      <c r="M144" s="64" t="inlineStr">
         <is>
           <t>ASN0003</t>
         </is>
@@ -6364,7 +6367,7 @@
       <c r="H145" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I145" s="11" t="inlineStr">
+      <c r="I145" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -6384,7 +6387,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M145" s="64" t="inlineStr">
+      <c r="M145" s="65" t="inlineStr">
         <is>
           <t>ASN0004</t>
         </is>
@@ -6432,7 +6435,7 @@
       <c r="H146" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I146" s="11" t="inlineStr">
+      <c r="I146" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -6452,7 +6455,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M146" s="64" t="inlineStr">
+      <c r="M146" s="65" t="inlineStr">
         <is>
           <t>ASN0005</t>
         </is>
@@ -6500,7 +6503,7 @@
       <c r="H147" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I147" s="11" t="inlineStr">
+      <c r="I147" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -6520,7 +6523,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M147" s="64" t="inlineStr">
+      <c r="M147" s="65" t="inlineStr">
         <is>
           <t>ASN0005</t>
         </is>
@@ -6568,7 +6571,7 @@
       <c r="H148" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I148" s="11" t="inlineStr">
+      <c r="I148" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -6588,7 +6591,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M148" s="64" t="inlineStr">
+      <c r="M148" s="65" t="inlineStr">
         <is>
           <t>ASN0005</t>
         </is>
@@ -6684,7 +6687,7 @@
           <t>9715300</t>
         </is>
       </c>
-      <c r="B155" s="63" t="inlineStr">
+      <c r="B155" s="64" t="inlineStr">
         <is>
           <t>CO-14101</t>
         </is>
@@ -6715,7 +6718,7 @@
       <c r="H155" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I155" s="11" t="inlineStr">
+      <c r="I155" s="56" t="inlineStr">
         <is>
           <t>6</t>
         </is>
@@ -6731,7 +6734,7 @@
           <t>9722D10</t>
         </is>
       </c>
-      <c r="B156" s="63" t="inlineStr">
+      <c r="B156" s="64" t="inlineStr">
         <is>
           <t>CO-14102</t>
         </is>
@@ -6762,7 +6765,7 @@
       <c r="H156" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I156" s="11" t="inlineStr">
+      <c r="I156" s="56" t="inlineStr">
         <is>
           <t>2</t>
         </is>
@@ -6778,7 +6781,7 @@
           <t>9722D10</t>
         </is>
       </c>
-      <c r="B157" s="63" t="inlineStr">
+      <c r="B157" s="64" t="inlineStr">
         <is>
           <t>CO-14103</t>
         </is>
@@ -6809,7 +6812,7 @@
       <c r="H157" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I157" s="11" t="inlineStr">
+      <c r="I157" s="56" t="inlineStr">
         <is>
           <t>6</t>
         </is>
@@ -6825,7 +6828,7 @@
           <t>9722D10</t>
         </is>
       </c>
-      <c r="B158" s="63" t="inlineStr">
+      <c r="B158" s="64" t="inlineStr">
         <is>
           <t>CO-14104</t>
         </is>
@@ -6856,7 +6859,7 @@
       <c r="H158" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I158" s="11" t="inlineStr">
+      <c r="I158" s="56" t="inlineStr">
         <is>
           <t>2</t>
         </is>
@@ -6872,7 +6875,7 @@
           <t>9715300</t>
         </is>
       </c>
-      <c r="B159" s="63" t="inlineStr">
+      <c r="B159" s="64" t="inlineStr">
         <is>
           <t>CO-14105</t>
         </is>
@@ -6903,7 +6906,7 @@
       <c r="H159" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I159" s="11" t="inlineStr">
+      <c r="I159" s="56" t="inlineStr">
         <is>
           <t>6</t>
         </is>
@@ -6919,7 +6922,7 @@
           <t>9715300</t>
         </is>
       </c>
-      <c r="B160" s="63" t="inlineStr">
+      <c r="B160" s="64" t="inlineStr">
         <is>
           <t>CO-14106</t>
         </is>
@@ -6950,7 +6953,7 @@
       <c r="H160" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="I160" s="11" t="inlineStr">
+      <c r="I160" s="56" t="inlineStr">
         <is>
           <t>6</t>
         </is>
@@ -6966,7 +6969,7 @@
           <t>9715300</t>
         </is>
       </c>
-      <c r="B161" s="63" t="inlineStr">
+      <c r="B161" s="64" t="inlineStr">
         <is>
           <t>CO-14107</t>
         </is>
@@ -6997,7 +7000,7 @@
       <c r="H161" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="I161" s="11" t="inlineStr">
+      <c r="I161" s="56" t="inlineStr">
         <is>
           <t>6</t>
         </is>
@@ -7013,7 +7016,7 @@
           <t>9811100</t>
         </is>
       </c>
-      <c r="B162" s="63" t="inlineStr">
+      <c r="B162" s="64" t="inlineStr">
         <is>
           <t>CO-14109</t>
         </is>
@@ -7044,7 +7047,7 @@
       <c r="H162" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I162" s="11" t="inlineStr">
+      <c r="I162" s="56" t="inlineStr">
         <is>
           <t>6</t>
         </is>
@@ -7060,7 +7063,7 @@
           <t>982200</t>
         </is>
       </c>
-      <c r="B163" s="63" t="inlineStr">
+      <c r="B163" s="64" t="inlineStr">
         <is>
           <t>CO-14110</t>
         </is>
@@ -7107,7 +7110,7 @@
           <t>9715300</t>
         </is>
       </c>
-      <c r="B164" s="63" t="inlineStr">
+      <c r="B164" s="64" t="inlineStr">
         <is>
           <t>CO-14112</t>
         </is>
@@ -7154,7 +7157,7 @@
           <t>9811100</t>
         </is>
       </c>
-      <c r="B165" s="63" t="inlineStr">
+      <c r="B165" s="64" t="inlineStr">
         <is>
           <t>CO-14113</t>
         </is>
@@ -7201,7 +7204,7 @@
           <t>982200</t>
         </is>
       </c>
-      <c r="B166" s="63" t="inlineStr">
+      <c r="B166" s="64" t="inlineStr">
         <is>
           <t>CO-14114</t>
         </is>
@@ -7248,7 +7251,7 @@
           <t>9722D10</t>
         </is>
       </c>
-      <c r="B167" s="63" t="inlineStr">
+      <c r="B167" s="64" t="inlineStr">
         <is>
           <t>CO-14111</t>
         </is>
@@ -7295,7 +7298,7 @@
           <t>9715300</t>
         </is>
       </c>
-      <c r="B168" s="63" t="inlineStr">
+      <c r="B168" s="64" t="inlineStr">
         <is>
           <t>CO-14115</t>
         </is>
@@ -7472,7 +7475,7 @@
       <c r="H175" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I175" s="11" t="inlineStr">
+      <c r="I175" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -7492,7 +7495,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M175" s="63" t="inlineStr">
+      <c r="M175" s="64" t="inlineStr">
         <is>
           <t>ASN0001</t>
         </is>
@@ -7540,7 +7543,7 @@
       <c r="H176" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I176" s="11" t="inlineStr">
+      <c r="I176" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -7608,7 +7611,7 @@
       <c r="H177" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I177" s="11" t="inlineStr">
+      <c r="I177" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -7628,7 +7631,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M177" s="63" t="inlineStr">
+      <c r="M177" s="64" t="inlineStr">
         <is>
           <t>ASN0002</t>
         </is>
@@ -7676,7 +7679,7 @@
       <c r="H178" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I178" s="11" t="inlineStr">
+      <c r="I178" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -7696,7 +7699,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M178" s="63" t="inlineStr">
+      <c r="M178" s="64" t="inlineStr">
         <is>
           <t>ASN0003</t>
         </is>
@@ -7744,7 +7747,7 @@
       <c r="H179" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="I179" s="11" t="inlineStr">
+      <c r="I179" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -7764,7 +7767,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M179" s="63" t="inlineStr">
+      <c r="M179" s="64" t="inlineStr">
         <is>
           <t>ASN0003</t>
         </is>
@@ -7812,7 +7815,7 @@
       <c r="H180" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="I180" s="11" t="inlineStr">
+      <c r="I180" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -7832,7 +7835,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M180" s="63" t="inlineStr">
+      <c r="M180" s="64" t="inlineStr">
         <is>
           <t>ASN0003</t>
         </is>
@@ -7880,7 +7883,7 @@
       <c r="H181" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I181" s="11" t="inlineStr">
+      <c r="I181" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -7900,7 +7903,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M181" s="63" t="inlineStr">
+      <c r="M181" s="64" t="inlineStr">
         <is>
           <t>ASN0003</t>
         </is>
@@ -7948,7 +7951,7 @@
       <c r="H182" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I182" s="11" t="inlineStr">
+      <c r="I182" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -7968,7 +7971,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M182" s="63" t="inlineStr">
+      <c r="M182" s="64" t="inlineStr">
         <is>
           <t>ASN0003</t>
         </is>
@@ -8016,7 +8019,7 @@
       <c r="H183" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I183" s="11" t="inlineStr">
+      <c r="I183" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -8036,7 +8039,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M183" s="63" t="inlineStr">
+      <c r="M183" s="64" t="inlineStr">
         <is>
           <t>ASN0004</t>
         </is>
@@ -8084,7 +8087,7 @@
       <c r="H184" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I184" s="11" t="inlineStr">
+      <c r="I184" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -8104,7 +8107,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M184" s="63" t="inlineStr">
+      <c r="M184" s="64" t="inlineStr">
         <is>
           <t>ASN0005</t>
         </is>
@@ -8152,7 +8155,7 @@
       <c r="H185" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I185" s="11" t="inlineStr">
+      <c r="I185" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -8172,7 +8175,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M185" s="63" t="inlineStr">
+      <c r="M185" s="64" t="inlineStr">
         <is>
           <t>ASN0005</t>
         </is>
@@ -8220,7 +8223,7 @@
       <c r="H186" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I186" s="11" t="inlineStr">
+      <c r="I186" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -8240,7 +8243,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M186" s="63" t="inlineStr">
+      <c r="M186" s="64" t="inlineStr">
         <is>
           <t>ASN0005</t>
         </is>
@@ -8519,7 +8522,7 @@
       <c r="H195" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I195" s="11" t="inlineStr">
+      <c r="I195" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -8539,7 +8542,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M195" s="63" t="inlineStr">
+      <c r="M195" s="64" t="inlineStr">
         <is>
           <t>ASN0001</t>
         </is>
@@ -8587,7 +8590,7 @@
       <c r="H196" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I196" s="11" t="inlineStr">
+      <c r="I196" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -8655,7 +8658,7 @@
       <c r="H197" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I197" s="11" t="inlineStr">
+      <c r="I197" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -8675,7 +8678,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M197" s="63" t="inlineStr">
+      <c r="M197" s="64" t="inlineStr">
         <is>
           <t>ASN0002</t>
         </is>
@@ -8723,7 +8726,7 @@
       <c r="H198" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I198" s="11" t="inlineStr">
+      <c r="I198" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -8743,7 +8746,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M198" s="63" t="inlineStr">
+      <c r="M198" s="64" t="inlineStr">
         <is>
           <t>ASN0003</t>
         </is>
@@ -8791,7 +8794,7 @@
       <c r="H199" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="I199" s="11" t="inlineStr">
+      <c r="I199" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -8811,7 +8814,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M199" s="63" t="inlineStr">
+      <c r="M199" s="64" t="inlineStr">
         <is>
           <t>ASN0003</t>
         </is>
@@ -8859,7 +8862,7 @@
       <c r="H200" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="I200" s="11" t="inlineStr">
+      <c r="I200" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -8879,7 +8882,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M200" s="63" t="inlineStr">
+      <c r="M200" s="64" t="inlineStr">
         <is>
           <t>ASN0003</t>
         </is>
@@ -8927,7 +8930,7 @@
       <c r="H201" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I201" s="11" t="inlineStr">
+      <c r="I201" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -8947,7 +8950,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M201" s="63" t="inlineStr">
+      <c r="M201" s="64" t="inlineStr">
         <is>
           <t>ASN0003</t>
         </is>
@@ -8995,7 +8998,7 @@
       <c r="H202" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I202" s="11" t="inlineStr">
+      <c r="I202" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -9015,7 +9018,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M202" s="63" t="inlineStr">
+      <c r="M202" s="64" t="inlineStr">
         <is>
           <t>ASN0003</t>
         </is>
@@ -9063,7 +9066,7 @@
       <c r="H203" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I203" s="11" t="inlineStr">
+      <c r="I203" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -9083,7 +9086,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M203" s="63" t="inlineStr">
+      <c r="M203" s="64" t="inlineStr">
         <is>
           <t>ASN0004</t>
         </is>
@@ -9131,7 +9134,7 @@
       <c r="H204" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I204" s="11" t="inlineStr">
+      <c r="I204" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -9151,7 +9154,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M204" s="63" t="inlineStr">
+      <c r="M204" s="64" t="inlineStr">
         <is>
           <t>ASN0005</t>
         </is>
@@ -9199,7 +9202,7 @@
       <c r="H205" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I205" s="11" t="inlineStr">
+      <c r="I205" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -9219,7 +9222,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M205" s="63" t="inlineStr">
+      <c r="M205" s="64" t="inlineStr">
         <is>
           <t>ASN0005</t>
         </is>
@@ -9267,7 +9270,7 @@
       <c r="H206" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I206" s="11" t="inlineStr">
+      <c r="I206" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -9287,7 +9290,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M206" s="63" t="inlineStr">
+      <c r="M206" s="64" t="inlineStr">
         <is>
           <t>ASN0005</t>
         </is>
@@ -9335,7 +9338,7 @@
       <c r="H207" s="15" t="n">
         <v>12</v>
       </c>
-      <c r="I207" s="11" t="inlineStr">
+      <c r="I207" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -9355,7 +9358,7 @@
           <t>N</t>
         </is>
       </c>
-      <c r="M207" s="64" t="inlineStr">
+      <c r="M207" s="65" t="inlineStr">
         <is>
           <t>ASN0006</t>
         </is>
@@ -9403,7 +9406,7 @@
       <c r="H208" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I208" s="11" t="inlineStr">
+      <c r="I208" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -9566,7 +9569,7 @@
       <c r="H215" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I215" s="11" t="inlineStr">
+      <c r="I215" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -9586,7 +9589,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M215" s="63" t="inlineStr">
+      <c r="M215" s="64" t="inlineStr">
         <is>
           <t>ASN0001</t>
         </is>
@@ -9634,7 +9637,7 @@
       <c r="H216" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I216" s="11" t="inlineStr">
+      <c r="I216" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -9702,7 +9705,7 @@
       <c r="H217" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I217" s="11" t="inlineStr">
+      <c r="I217" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -9722,7 +9725,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M217" s="63" t="inlineStr">
+      <c r="M217" s="64" t="inlineStr">
         <is>
           <t>ASN0002</t>
         </is>
@@ -9770,7 +9773,7 @@
       <c r="H218" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I218" s="11" t="inlineStr">
+      <c r="I218" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -9790,7 +9793,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M218" s="63" t="inlineStr">
+      <c r="M218" s="64" t="inlineStr">
         <is>
           <t>ASN0003</t>
         </is>
@@ -9838,7 +9841,7 @@
       <c r="H219" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="I219" s="11" t="inlineStr">
+      <c r="I219" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -9858,7 +9861,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M219" s="63" t="inlineStr">
+      <c r="M219" s="64" t="inlineStr">
         <is>
           <t>ASN0003</t>
         </is>
@@ -9906,7 +9909,7 @@
       <c r="H220" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="I220" s="11" t="inlineStr">
+      <c r="I220" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -9926,7 +9929,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M220" s="63" t="inlineStr">
+      <c r="M220" s="64" t="inlineStr">
         <is>
           <t>ASN0003</t>
         </is>
@@ -9974,7 +9977,7 @@
       <c r="H221" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I221" s="11" t="inlineStr">
+      <c r="I221" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -9994,7 +9997,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M221" s="63" t="inlineStr">
+      <c r="M221" s="64" t="inlineStr">
         <is>
           <t>ASN0003</t>
         </is>
@@ -10042,7 +10045,7 @@
       <c r="H222" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I222" s="11" t="inlineStr">
+      <c r="I222" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -10062,7 +10065,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M222" s="63" t="inlineStr">
+      <c r="M222" s="64" t="inlineStr">
         <is>
           <t>ASN0003</t>
         </is>
@@ -10110,7 +10113,7 @@
       <c r="H223" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I223" s="11" t="inlineStr">
+      <c r="I223" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -10130,7 +10133,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M223" s="63" t="inlineStr">
+      <c r="M223" s="64" t="inlineStr">
         <is>
           <t>ASN0004</t>
         </is>
@@ -10178,7 +10181,7 @@
       <c r="H224" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I224" s="11" t="inlineStr">
+      <c r="I224" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -10198,7 +10201,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M224" s="63" t="inlineStr">
+      <c r="M224" s="64" t="inlineStr">
         <is>
           <t>ASN0005</t>
         </is>
@@ -10246,7 +10249,7 @@
       <c r="H225" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I225" s="11" t="inlineStr">
+      <c r="I225" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -10266,7 +10269,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M225" s="63" t="inlineStr">
+      <c r="M225" s="64" t="inlineStr">
         <is>
           <t>ASN0005</t>
         </is>
@@ -10314,7 +10317,7 @@
       <c r="H226" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I226" s="11" t="inlineStr">
+      <c r="I226" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -10334,7 +10337,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M226" s="63" t="inlineStr">
+      <c r="M226" s="64" t="inlineStr">
         <is>
           <t>ASN0005</t>
         </is>
@@ -10382,7 +10385,7 @@
       <c r="H227" s="15" t="n">
         <v>12</v>
       </c>
-      <c r="I227" s="11" t="inlineStr">
+      <c r="I227" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -10402,7 +10405,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M227" s="56" t="inlineStr">
+      <c r="M227" s="57" t="inlineStr">
         <is>
           <t>ASN0006, ASN0007</t>
         </is>
@@ -10450,7 +10453,7 @@
       <c r="H228" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I228" s="11" t="inlineStr">
+      <c r="I228" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -10566,7 +10569,7 @@
           <t>9715300</t>
         </is>
       </c>
-      <c r="B235" s="63" t="inlineStr">
+      <c r="B235" s="64" t="inlineStr">
         <is>
           <t>CO-14101</t>
         </is>
@@ -10597,7 +10600,7 @@
       <c r="H235" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I235" s="11" t="inlineStr">
+      <c r="I235" s="56" t="inlineStr">
         <is>
           <t>6</t>
         </is>
@@ -10613,7 +10616,7 @@
           <t>9722D10</t>
         </is>
       </c>
-      <c r="B236" s="63" t="inlineStr">
+      <c r="B236" s="64" t="inlineStr">
         <is>
           <t>CO-14102</t>
         </is>
@@ -10644,7 +10647,7 @@
       <c r="H236" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I236" s="11" t="inlineStr">
+      <c r="I236" s="56" t="inlineStr">
         <is>
           <t>2</t>
         </is>
@@ -10660,7 +10663,7 @@
           <t>9722D10</t>
         </is>
       </c>
-      <c r="B237" s="63" t="inlineStr">
+      <c r="B237" s="64" t="inlineStr">
         <is>
           <t>CO-14103</t>
         </is>
@@ -10691,7 +10694,7 @@
       <c r="H237" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I237" s="11" t="inlineStr">
+      <c r="I237" s="56" t="inlineStr">
         <is>
           <t>6</t>
         </is>
@@ -10707,7 +10710,7 @@
           <t>9722D10</t>
         </is>
       </c>
-      <c r="B238" s="63" t="inlineStr">
+      <c r="B238" s="64" t="inlineStr">
         <is>
           <t>CO-14104</t>
         </is>
@@ -10738,7 +10741,7 @@
       <c r="H238" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I238" s="11" t="inlineStr">
+      <c r="I238" s="56" t="inlineStr">
         <is>
           <t>2</t>
         </is>
@@ -10754,7 +10757,7 @@
           <t>9715300</t>
         </is>
       </c>
-      <c r="B239" s="63" t="inlineStr">
+      <c r="B239" s="64" t="inlineStr">
         <is>
           <t>CO-14105</t>
         </is>
@@ -10785,7 +10788,7 @@
       <c r="H239" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I239" s="11" t="inlineStr">
+      <c r="I239" s="56" t="inlineStr">
         <is>
           <t>6</t>
         </is>
@@ -10801,7 +10804,7 @@
           <t>9715300</t>
         </is>
       </c>
-      <c r="B240" s="63" t="inlineStr">
+      <c r="B240" s="64" t="inlineStr">
         <is>
           <t>CO-14106</t>
         </is>
@@ -10832,7 +10835,7 @@
       <c r="H240" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="I240" s="11" t="inlineStr">
+      <c r="I240" s="56" t="inlineStr">
         <is>
           <t>6</t>
         </is>
@@ -10848,7 +10851,7 @@
           <t>9715300</t>
         </is>
       </c>
-      <c r="B241" s="63" t="inlineStr">
+      <c r="B241" s="64" t="inlineStr">
         <is>
           <t>CO-14107</t>
         </is>
@@ -10879,7 +10882,7 @@
       <c r="H241" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="I241" s="11" t="inlineStr">
+      <c r="I241" s="56" t="inlineStr">
         <is>
           <t>6</t>
         </is>
@@ -10895,7 +10898,7 @@
           <t>9811100</t>
         </is>
       </c>
-      <c r="B242" s="63" t="inlineStr">
+      <c r="B242" s="64" t="inlineStr">
         <is>
           <t>CO-14109</t>
         </is>
@@ -10926,7 +10929,7 @@
       <c r="H242" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I242" s="11" t="inlineStr">
+      <c r="I242" s="56" t="inlineStr">
         <is>
           <t>6</t>
         </is>
@@ -10942,7 +10945,7 @@
           <t>982200</t>
         </is>
       </c>
-      <c r="B243" s="63" t="inlineStr">
+      <c r="B243" s="64" t="inlineStr">
         <is>
           <t>CO-14110</t>
         </is>
@@ -10973,7 +10976,7 @@
       <c r="H243" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I243" s="11" t="inlineStr">
+      <c r="I243" s="56" t="inlineStr">
         <is>
           <t>6</t>
         </is>
@@ -10989,7 +10992,7 @@
           <t>9715300</t>
         </is>
       </c>
-      <c r="B244" s="63" t="inlineStr">
+      <c r="B244" s="64" t="inlineStr">
         <is>
           <t>CO-14112</t>
         </is>
@@ -11020,7 +11023,7 @@
       <c r="H244" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I244" s="11" t="inlineStr">
+      <c r="I244" s="56" t="inlineStr">
         <is>
           <t>6</t>
         </is>
@@ -11036,7 +11039,7 @@
           <t>9811100</t>
         </is>
       </c>
-      <c r="B245" s="63" t="inlineStr">
+      <c r="B245" s="64" t="inlineStr">
         <is>
           <t>CO-14113</t>
         </is>
@@ -11067,7 +11070,7 @@
       <c r="H245" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I245" s="11" t="inlineStr">
+      <c r="I245" s="56" t="inlineStr">
         <is>
           <t>6</t>
         </is>
@@ -11083,7 +11086,7 @@
           <t>982200</t>
         </is>
       </c>
-      <c r="B246" s="63" t="inlineStr">
+      <c r="B246" s="64" t="inlineStr">
         <is>
           <t>CO-14114</t>
         </is>
@@ -11114,7 +11117,7 @@
       <c r="H246" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I246" s="11" t="inlineStr">
+      <c r="I246" s="56" t="inlineStr">
         <is>
           <t>6</t>
         </is>
@@ -11130,7 +11133,7 @@
           <t>9722D10</t>
         </is>
       </c>
-      <c r="B247" s="63" t="inlineStr">
+      <c r="B247" s="64" t="inlineStr">
         <is>
           <t>CO-14111</t>
         </is>
@@ -11181,7 +11184,7 @@
           <t>9715300</t>
         </is>
       </c>
-      <c r="B248" s="63" t="inlineStr">
+      <c r="B248" s="64" t="inlineStr">
         <is>
           <t>CO-14115</t>
         </is>
@@ -11232,7 +11235,7 @@
           <t>9715300</t>
         </is>
       </c>
-      <c r="B249" s="63" t="inlineStr">
+      <c r="B249" s="64" t="inlineStr">
         <is>
           <t>CO-14115</t>
         </is>
@@ -11250,7 +11253,7 @@
           <t>001</t>
         </is>
       </c>
-      <c r="F249" s="56" t="inlineStr">
+      <c r="F249" s="57" t="inlineStr">
         <is>
           <t>0000002</t>
         </is>
@@ -11409,7 +11412,7 @@
       <c r="H256" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I256" s="11" t="inlineStr">
+      <c r="I256" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -11429,7 +11432,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M256" s="63" t="inlineStr">
+      <c r="M256" s="64" t="inlineStr">
         <is>
           <t>ASN0001</t>
         </is>
@@ -11477,7 +11480,7 @@
       <c r="H257" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I257" s="11" t="inlineStr">
+      <c r="I257" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -11545,7 +11548,7 @@
       <c r="H258" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I258" s="11" t="inlineStr">
+      <c r="I258" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -11565,7 +11568,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M258" s="63" t="inlineStr">
+      <c r="M258" s="64" t="inlineStr">
         <is>
           <t>ASN0002</t>
         </is>
@@ -11613,7 +11616,7 @@
       <c r="H259" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I259" s="11" t="inlineStr">
+      <c r="I259" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -11633,7 +11636,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M259" s="63" t="inlineStr">
+      <c r="M259" s="64" t="inlineStr">
         <is>
           <t>ASN0003</t>
         </is>
@@ -11681,7 +11684,7 @@
       <c r="H260" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="I260" s="11" t="inlineStr">
+      <c r="I260" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -11701,7 +11704,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M260" s="63" t="inlineStr">
+      <c r="M260" s="64" t="inlineStr">
         <is>
           <t>ASN0003</t>
         </is>
@@ -11749,7 +11752,7 @@
       <c r="H261" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="I261" s="11" t="inlineStr">
+      <c r="I261" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -11769,7 +11772,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M261" s="63" t="inlineStr">
+      <c r="M261" s="64" t="inlineStr">
         <is>
           <t>ASN0003</t>
         </is>
@@ -11817,7 +11820,7 @@
       <c r="H262" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I262" s="11" t="inlineStr">
+      <c r="I262" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -11837,7 +11840,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M262" s="63" t="inlineStr">
+      <c r="M262" s="64" t="inlineStr">
         <is>
           <t>ASN0003</t>
         </is>
@@ -11885,7 +11888,7 @@
       <c r="H263" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I263" s="11" t="inlineStr">
+      <c r="I263" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -11905,7 +11908,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M263" s="63" t="inlineStr">
+      <c r="M263" s="64" t="inlineStr">
         <is>
           <t>ASN0003</t>
         </is>
@@ -11953,7 +11956,7 @@
       <c r="H264" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I264" s="11" t="inlineStr">
+      <c r="I264" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -11973,7 +11976,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M264" s="63" t="inlineStr">
+      <c r="M264" s="64" t="inlineStr">
         <is>
           <t>ASN0004</t>
         </is>
@@ -12021,7 +12024,7 @@
       <c r="H265" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I265" s="11" t="inlineStr">
+      <c r="I265" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -12041,7 +12044,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M265" s="63" t="inlineStr">
+      <c r="M265" s="64" t="inlineStr">
         <is>
           <t>ASN0005</t>
         </is>
@@ -12089,7 +12092,7 @@
       <c r="H266" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I266" s="11" t="inlineStr">
+      <c r="I266" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -12109,7 +12112,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M266" s="63" t="inlineStr">
+      <c r="M266" s="64" t="inlineStr">
         <is>
           <t>ASN0005</t>
         </is>
@@ -12157,7 +12160,7 @@
       <c r="H267" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I267" s="11" t="inlineStr">
+      <c r="I267" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -12177,7 +12180,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M267" s="63" t="inlineStr">
+      <c r="M267" s="64" t="inlineStr">
         <is>
           <t>ASN0005</t>
         </is>
@@ -12225,7 +12228,7 @@
       <c r="H268" s="55" t="n">
         <v>6</v>
       </c>
-      <c r="I268" s="11" t="inlineStr">
+      <c r="I268" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -12361,7 +12364,7 @@
       <c r="H270" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I270" s="11" t="inlineStr">
+      <c r="I270" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -12524,7 +12527,7 @@
       <c r="H277" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I277" s="11" t="inlineStr">
+      <c r="I277" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -12544,7 +12547,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M277" s="63" t="inlineStr">
+      <c r="M277" s="64" t="inlineStr">
         <is>
           <t>ASN0001</t>
         </is>
@@ -12592,7 +12595,7 @@
       <c r="H278" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I278" s="11" t="inlineStr">
+      <c r="I278" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -12660,7 +12663,7 @@
       <c r="H279" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I279" s="11" t="inlineStr">
+      <c r="I279" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -12680,7 +12683,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M279" s="63" t="inlineStr">
+      <c r="M279" s="64" t="inlineStr">
         <is>
           <t>ASN0002</t>
         </is>
@@ -12728,7 +12731,7 @@
       <c r="H280" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I280" s="11" t="inlineStr">
+      <c r="I280" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -12748,7 +12751,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M280" s="63" t="inlineStr">
+      <c r="M280" s="64" t="inlineStr">
         <is>
           <t>ASN0003</t>
         </is>
@@ -12796,7 +12799,7 @@
       <c r="H281" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="I281" s="11" t="inlineStr">
+      <c r="I281" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -12816,7 +12819,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M281" s="63" t="inlineStr">
+      <c r="M281" s="64" t="inlineStr">
         <is>
           <t>ASN0003</t>
         </is>
@@ -12864,7 +12867,7 @@
       <c r="H282" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="I282" s="11" t="inlineStr">
+      <c r="I282" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -12884,7 +12887,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M282" s="63" t="inlineStr">
+      <c r="M282" s="64" t="inlineStr">
         <is>
           <t>ASN0003</t>
         </is>
@@ -12932,7 +12935,7 @@
       <c r="H283" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I283" s="11" t="inlineStr">
+      <c r="I283" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -12952,7 +12955,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M283" s="63" t="inlineStr">
+      <c r="M283" s="64" t="inlineStr">
         <is>
           <t>ASN0003</t>
         </is>
@@ -13000,7 +13003,7 @@
       <c r="H284" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I284" s="11" t="inlineStr">
+      <c r="I284" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -13020,7 +13023,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M284" s="63" t="inlineStr">
+      <c r="M284" s="64" t="inlineStr">
         <is>
           <t>ASN0003</t>
         </is>
@@ -13068,7 +13071,7 @@
       <c r="H285" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I285" s="11" t="inlineStr">
+      <c r="I285" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -13088,7 +13091,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M285" s="63" t="inlineStr">
+      <c r="M285" s="64" t="inlineStr">
         <is>
           <t>ASN0004</t>
         </is>
@@ -13136,7 +13139,7 @@
       <c r="H286" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I286" s="11" t="inlineStr">
+      <c r="I286" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -13156,7 +13159,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M286" s="63" t="inlineStr">
+      <c r="M286" s="64" t="inlineStr">
         <is>
           <t>ASN0005</t>
         </is>
@@ -13204,7 +13207,7 @@
       <c r="H287" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I287" s="11" t="inlineStr">
+      <c r="I287" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -13224,7 +13227,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M287" s="63" t="inlineStr">
+      <c r="M287" s="64" t="inlineStr">
         <is>
           <t>ASN0005</t>
         </is>
@@ -13272,7 +13275,7 @@
       <c r="H288" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I288" s="11" t="inlineStr">
+      <c r="I288" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -13292,7 +13295,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M288" s="63" t="inlineStr">
+      <c r="M288" s="64" t="inlineStr">
         <is>
           <t>ASN0005</t>
         </is>
@@ -13340,7 +13343,7 @@
       <c r="H289" s="55" t="n">
         <v>6</v>
       </c>
-      <c r="I289" s="11" t="inlineStr">
+      <c r="I289" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -13360,7 +13363,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M289" s="64" t="inlineStr">
+      <c r="M289" s="65" t="inlineStr">
         <is>
           <t>ASN0006</t>
         </is>
@@ -13428,7 +13431,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M290" s="63" t="inlineStr">
+      <c r="M290" s="64" t="inlineStr">
         <is>
           <t>ASN0007</t>
         </is>
@@ -13476,7 +13479,7 @@
       <c r="H291" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I291" s="11" t="inlineStr">
+      <c r="I291" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -13639,7 +13642,7 @@
       <c r="H298" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I298" s="11" t="inlineStr">
+      <c r="I298" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -13659,7 +13662,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M298" s="63" t="inlineStr">
+      <c r="M298" s="64" t="inlineStr">
         <is>
           <t>ASN0001</t>
         </is>
@@ -13707,7 +13710,7 @@
       <c r="H299" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I299" s="11" t="inlineStr">
+      <c r="I299" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -13775,7 +13778,7 @@
       <c r="H300" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I300" s="11" t="inlineStr">
+      <c r="I300" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -13795,7 +13798,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M300" s="63" t="inlineStr">
+      <c r="M300" s="64" t="inlineStr">
         <is>
           <t>ASN0002</t>
         </is>
@@ -13843,7 +13846,7 @@
       <c r="H301" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I301" s="11" t="inlineStr">
+      <c r="I301" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -13863,7 +13866,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M301" s="63" t="inlineStr">
+      <c r="M301" s="64" t="inlineStr">
         <is>
           <t>ASN0003</t>
         </is>
@@ -13911,7 +13914,7 @@
       <c r="H302" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="I302" s="11" t="inlineStr">
+      <c r="I302" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -13931,7 +13934,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M302" s="63" t="inlineStr">
+      <c r="M302" s="64" t="inlineStr">
         <is>
           <t>ASN0003</t>
         </is>
@@ -13979,7 +13982,7 @@
       <c r="H303" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="I303" s="11" t="inlineStr">
+      <c r="I303" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -13999,7 +14002,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M303" s="63" t="inlineStr">
+      <c r="M303" s="64" t="inlineStr">
         <is>
           <t>ASN0003</t>
         </is>
@@ -14047,7 +14050,7 @@
       <c r="H304" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I304" s="11" t="inlineStr">
+      <c r="I304" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -14067,7 +14070,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M304" s="56" t="inlineStr">
+      <c r="M304" s="57" t="inlineStr">
         <is>
           <t>NULL</t>
         </is>
@@ -14115,7 +14118,7 @@
       <c r="H305" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I305" s="11" t="inlineStr">
+      <c r="I305" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -14135,7 +14138,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M305" s="63" t="inlineStr">
+      <c r="M305" s="64" t="inlineStr">
         <is>
           <t>ASN0003</t>
         </is>
@@ -14183,7 +14186,7 @@
       <c r="H306" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I306" s="11" t="inlineStr">
+      <c r="I306" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -14203,7 +14206,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M306" s="63" t="inlineStr">
+      <c r="M306" s="64" t="inlineStr">
         <is>
           <t>ASN0004</t>
         </is>
@@ -14251,7 +14254,7 @@
       <c r="H307" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I307" s="11" t="inlineStr">
+      <c r="I307" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -14271,7 +14274,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M307" s="63" t="inlineStr">
+      <c r="M307" s="64" t="inlineStr">
         <is>
           <t>ASN0005</t>
         </is>
@@ -14319,7 +14322,7 @@
       <c r="H308" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I308" s="11" t="inlineStr">
+      <c r="I308" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -14339,7 +14342,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M308" s="63" t="inlineStr">
+      <c r="M308" s="64" t="inlineStr">
         <is>
           <t>ASN0005</t>
         </is>
@@ -14387,7 +14390,7 @@
       <c r="H309" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I309" s="11" t="inlineStr">
+      <c r="I309" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -14407,7 +14410,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M309" s="63" t="inlineStr">
+      <c r="M309" s="64" t="inlineStr">
         <is>
           <t>ASN0005</t>
         </is>
@@ -14455,7 +14458,7 @@
       <c r="H310" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I310" s="11" t="inlineStr">
+      <c r="I310" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -14475,7 +14478,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M310" s="63" t="inlineStr">
+      <c r="M310" s="64" t="inlineStr">
         <is>
           <t>ASN0006</t>
         </is>
@@ -14523,7 +14526,7 @@
       <c r="H311" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I311" s="11" t="inlineStr">
+      <c r="I311" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -14543,7 +14546,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M311" s="63" t="inlineStr">
+      <c r="M311" s="64" t="inlineStr">
         <is>
           <t>ASN0007</t>
         </is>
@@ -14591,7 +14594,7 @@
       <c r="H312" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I312" s="11" t="inlineStr">
+      <c r="I312" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -14611,7 +14614,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M312" s="64" t="inlineStr">
+      <c r="M312" s="65" t="inlineStr">
         <is>
           <t>ASN0003</t>
         </is>
@@ -14707,7 +14710,7 @@
           <t>9715300</t>
         </is>
       </c>
-      <c r="B319" s="63" t="inlineStr">
+      <c r="B319" s="64" t="inlineStr">
         <is>
           <t>CO-14101</t>
         </is>
@@ -14738,7 +14741,7 @@
       <c r="H319" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I319" s="11" t="inlineStr">
+      <c r="I319" s="56" t="inlineStr">
         <is>
           <t>6</t>
         </is>
@@ -14754,7 +14757,7 @@
           <t>9722D10</t>
         </is>
       </c>
-      <c r="B320" s="63" t="inlineStr">
+      <c r="B320" s="64" t="inlineStr">
         <is>
           <t>CO-14102</t>
         </is>
@@ -14785,7 +14788,7 @@
       <c r="H320" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I320" s="11" t="inlineStr">
+      <c r="I320" s="56" t="inlineStr">
         <is>
           <t>2</t>
         </is>
@@ -14801,7 +14804,7 @@
           <t>9722D10</t>
         </is>
       </c>
-      <c r="B321" s="63" t="inlineStr">
+      <c r="B321" s="64" t="inlineStr">
         <is>
           <t>CO-14103</t>
         </is>
@@ -14832,7 +14835,7 @@
       <c r="H321" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I321" s="11" t="inlineStr">
+      <c r="I321" s="56" t="inlineStr">
         <is>
           <t>6</t>
         </is>
@@ -14848,7 +14851,7 @@
           <t>9722D10</t>
         </is>
       </c>
-      <c r="B322" s="63" t="inlineStr">
+      <c r="B322" s="64" t="inlineStr">
         <is>
           <t>CO-14104</t>
         </is>
@@ -14879,7 +14882,7 @@
       <c r="H322" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I322" s="11" t="inlineStr">
+      <c r="I322" s="56" t="inlineStr">
         <is>
           <t>2</t>
         </is>
@@ -14895,7 +14898,7 @@
           <t>9715300</t>
         </is>
       </c>
-      <c r="B323" s="63" t="inlineStr">
+      <c r="B323" s="64" t="inlineStr">
         <is>
           <t>CO-14105</t>
         </is>
@@ -14926,7 +14929,7 @@
       <c r="H323" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I323" s="11" t="inlineStr">
+      <c r="I323" s="56" t="inlineStr">
         <is>
           <t>6</t>
         </is>
@@ -14942,7 +14945,7 @@
           <t>9715300</t>
         </is>
       </c>
-      <c r="B324" s="63" t="inlineStr">
+      <c r="B324" s="64" t="inlineStr">
         <is>
           <t>CO-14106</t>
         </is>
@@ -14973,7 +14976,7 @@
       <c r="H324" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="I324" s="11" t="inlineStr">
+      <c r="I324" s="56" t="inlineStr">
         <is>
           <t>6</t>
         </is>
@@ -14989,7 +14992,7 @@
           <t>9715300</t>
         </is>
       </c>
-      <c r="B325" s="63" t="inlineStr">
+      <c r="B325" s="64" t="inlineStr">
         <is>
           <t>CO-14107</t>
         </is>
@@ -15020,7 +15023,7 @@
       <c r="H325" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="I325" s="11" t="inlineStr">
+      <c r="I325" s="56" t="inlineStr">
         <is>
           <t>6</t>
         </is>
@@ -15036,7 +15039,7 @@
           <t>9811100</t>
         </is>
       </c>
-      <c r="B326" s="63" t="inlineStr">
+      <c r="B326" s="64" t="inlineStr">
         <is>
           <t>CO-14109</t>
         </is>
@@ -15067,7 +15070,7 @@
       <c r="H326" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I326" s="11" t="inlineStr">
+      <c r="I326" s="56" t="inlineStr">
         <is>
           <t>6</t>
         </is>
@@ -15083,7 +15086,7 @@
           <t>982200</t>
         </is>
       </c>
-      <c r="B327" s="63" t="inlineStr">
+      <c r="B327" s="64" t="inlineStr">
         <is>
           <t>CO-14110</t>
         </is>
@@ -15114,7 +15117,7 @@
       <c r="H327" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I327" s="11" t="inlineStr">
+      <c r="I327" s="56" t="inlineStr">
         <is>
           <t>6</t>
         </is>
@@ -15130,7 +15133,7 @@
           <t>9715300</t>
         </is>
       </c>
-      <c r="B328" s="63" t="inlineStr">
+      <c r="B328" s="64" t="inlineStr">
         <is>
           <t>CO-14112</t>
         </is>
@@ -15161,7 +15164,7 @@
       <c r="H328" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I328" s="11" t="inlineStr">
+      <c r="I328" s="56" t="inlineStr">
         <is>
           <t>6</t>
         </is>
@@ -15177,7 +15180,7 @@
           <t>9811100</t>
         </is>
       </c>
-      <c r="B329" s="63" t="inlineStr">
+      <c r="B329" s="64" t="inlineStr">
         <is>
           <t>CO-14113</t>
         </is>
@@ -15208,7 +15211,7 @@
       <c r="H329" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I329" s="11" t="inlineStr">
+      <c r="I329" s="56" t="inlineStr">
         <is>
           <t>6</t>
         </is>
@@ -15224,7 +15227,7 @@
           <t>982200</t>
         </is>
       </c>
-      <c r="B330" s="63" t="inlineStr">
+      <c r="B330" s="64" t="inlineStr">
         <is>
           <t>CO-14114</t>
         </is>
@@ -15255,7 +15258,7 @@
       <c r="H330" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I330" s="11" t="inlineStr">
+      <c r="I330" s="56" t="inlineStr">
         <is>
           <t>6</t>
         </is>
@@ -15271,7 +15274,7 @@
           <t>9722D10</t>
         </is>
       </c>
-      <c r="B331" s="63" t="inlineStr">
+      <c r="B331" s="64" t="inlineStr">
         <is>
           <t>CO-14111</t>
         </is>
@@ -15302,7 +15305,7 @@
       <c r="H331" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I331" s="11" t="inlineStr">
+      <c r="I331" s="56" t="inlineStr">
         <is>
           <t>6</t>
         </is>
@@ -15318,7 +15321,7 @@
           <t>9715300</t>
         </is>
       </c>
-      <c r="B332" s="63" t="inlineStr">
+      <c r="B332" s="64" t="inlineStr">
         <is>
           <t>CO-14115</t>
         </is>
@@ -15349,7 +15352,7 @@
       <c r="H332" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I332" s="11" t="inlineStr">
+      <c r="I332" s="56" t="inlineStr">
         <is>
           <t>6</t>
         </is>
@@ -15365,7 +15368,7 @@
           <t>9715300</t>
         </is>
       </c>
-      <c r="B333" s="63" t="inlineStr">
+      <c r="B333" s="64" t="inlineStr">
         <is>
           <t>CO-14115</t>
         </is>
@@ -15542,7 +15545,7 @@
       <c r="H340" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I340" s="11" t="inlineStr">
+      <c r="I340" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -15562,7 +15565,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M340" s="63" t="inlineStr">
+      <c r="M340" s="64" t="inlineStr">
         <is>
           <t>ASN0001</t>
         </is>
@@ -15610,7 +15613,7 @@
       <c r="H341" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I341" s="11" t="inlineStr">
+      <c r="I341" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -15678,7 +15681,7 @@
       <c r="H342" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I342" s="11" t="inlineStr">
+      <c r="I342" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -15698,7 +15701,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M342" s="63" t="inlineStr">
+      <c r="M342" s="64" t="inlineStr">
         <is>
           <t>ASN0002</t>
         </is>
@@ -15746,7 +15749,7 @@
       <c r="H343" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I343" s="11" t="inlineStr">
+      <c r="I343" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -15766,7 +15769,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M343" s="63" t="inlineStr">
+      <c r="M343" s="64" t="inlineStr">
         <is>
           <t>ASN0003</t>
         </is>
@@ -15814,7 +15817,7 @@
       <c r="H344" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="I344" s="11" t="inlineStr">
+      <c r="I344" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -15834,7 +15837,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M344" s="63" t="inlineStr">
+      <c r="M344" s="64" t="inlineStr">
         <is>
           <t>ASN0003</t>
         </is>
@@ -15882,7 +15885,7 @@
       <c r="H345" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="I345" s="11" t="inlineStr">
+      <c r="I345" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -15902,7 +15905,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M345" s="63" t="inlineStr">
+      <c r="M345" s="64" t="inlineStr">
         <is>
           <t>ASN0003</t>
         </is>
@@ -15950,7 +15953,7 @@
       <c r="H346" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I346" s="11" t="inlineStr">
+      <c r="I346" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -16018,7 +16021,7 @@
       <c r="H347" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I347" s="11" t="inlineStr">
+      <c r="I347" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -16038,7 +16041,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M347" s="63" t="inlineStr">
+      <c r="M347" s="64" t="inlineStr">
         <is>
           <t>ASN0003</t>
         </is>
@@ -16086,7 +16089,7 @@
       <c r="H348" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I348" s="11" t="inlineStr">
+      <c r="I348" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -16106,7 +16109,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M348" s="63" t="inlineStr">
+      <c r="M348" s="64" t="inlineStr">
         <is>
           <t>ASN0004</t>
         </is>
@@ -16154,7 +16157,7 @@
       <c r="H349" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I349" s="11" t="inlineStr">
+      <c r="I349" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -16174,7 +16177,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M349" s="63" t="inlineStr">
+      <c r="M349" s="64" t="inlineStr">
         <is>
           <t>ASN0005</t>
         </is>
@@ -16222,7 +16225,7 @@
       <c r="H350" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I350" s="11" t="inlineStr">
+      <c r="I350" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -16242,7 +16245,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M350" s="63" t="inlineStr">
+      <c r="M350" s="64" t="inlineStr">
         <is>
           <t>ASN0005</t>
         </is>
@@ -16290,7 +16293,7 @@
       <c r="H351" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I351" s="11" t="inlineStr">
+      <c r="I351" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -16310,7 +16313,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M351" s="63" t="inlineStr">
+      <c r="M351" s="64" t="inlineStr">
         <is>
           <t>ASN0005</t>
         </is>
@@ -16358,7 +16361,7 @@
       <c r="H352" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I352" s="11" t="inlineStr">
+      <c r="I352" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -16378,7 +16381,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M352" s="63" t="inlineStr">
+      <c r="M352" s="64" t="inlineStr">
         <is>
           <t>ASN0006</t>
         </is>
@@ -16426,7 +16429,7 @@
       <c r="H353" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I353" s="11" t="inlineStr">
+      <c r="I353" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -16446,7 +16449,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M353" s="63" t="inlineStr">
+      <c r="M353" s="64" t="inlineStr">
         <is>
           <t>ASN0007</t>
         </is>
@@ -16494,7 +16497,7 @@
       <c r="H354" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="I354" s="11" t="inlineStr">
+      <c r="I354" s="56" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -16514,7 +16517,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M354" s="63" t="inlineStr">
+      <c r="M354" s="64" t="inlineStr">
         <is>
           <t>ASN0003</t>
         </is>
@@ -16751,7 +16754,7 @@
   <sheetData>
     <row r="1"/>
     <row r="2" ht="14" customHeight="1" s="26">
-      <c r="B2" s="57" t="inlineStr">
+      <c r="B2" s="58" t="inlineStr">
         <is>
           <t>Cek PO per customer order date (1 order date = 1 PO, PO_DT = order date + 1)</t>
         </is>
@@ -16800,7 +16803,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="B4" s="65" t="n">
+      <c r="B4" s="66" t="n">
         <v>46310</v>
       </c>
       <c r="C4" s="46" t="n">
@@ -16809,12 +16812,12 @@
       <c r="D4" s="46" t="n">
         <v>12</v>
       </c>
-      <c r="E4" s="66" t="inlineStr">
+      <c r="E4" s="67" t="inlineStr">
         <is>
           <t>T0409011</t>
         </is>
       </c>
-      <c r="F4" s="65" t="n">
+      <c r="F4" s="66" t="n">
         <v>46311</v>
       </c>
       <c r="G4" s="46" t="n">
@@ -16832,7 +16835,7 @@
       </c>
     </row>
     <row r="5" ht="40" customHeight="1" s="26">
-      <c r="B5" s="65" t="n">
+      <c r="B5" s="66" t="n">
         <v>46311</v>
       </c>
       <c r="C5" s="46" t="n">
@@ -16841,12 +16844,12 @@
       <c r="D5" s="46" t="n">
         <v>6</v>
       </c>
-      <c r="E5" s="66" t="inlineStr">
+      <c r="E5" s="67" t="inlineStr">
         <is>
           <t>T0409012</t>
         </is>
       </c>
-      <c r="F5" s="65" t="n">
+      <c r="F5" s="66" t="n">
         <v>46312</v>
       </c>
       <c r="G5" s="46" t="n">
@@ -16864,7 +16867,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="65" t="n">
+      <c r="B6" s="66" t="n">
         <v>46312</v>
       </c>
       <c r="C6" s="46" t="n">
@@ -16873,30 +16876,30 @@
       <c r="D6" s="46" t="n">
         <v>30</v>
       </c>
-      <c r="E6" s="66" t="inlineStr">
+      <c r="E6" s="67" t="inlineStr">
         <is>
           <t>T0409013</t>
         </is>
       </c>
-      <c r="F6" s="65" t="n">
+      <c r="F6" s="66" t="n">
         <v>46313</v>
       </c>
       <c r="G6" s="46" t="n">
         <v>18</v>
       </c>
-      <c r="H6" s="59" t="inlineStr">
+      <c r="H6" s="60" t="inlineStr">
         <is>
           <t>ABNORMAL (kurang 12)</t>
         </is>
       </c>
-      <c r="I6" s="66" t="inlineStr">
+      <c r="I6" s="67" t="inlineStr">
         <is>
           <t>T0409014 (12)</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="65" t="n">
+      <c r="B7" s="66" t="n">
         <v>46313</v>
       </c>
       <c r="C7" s="46" t="n">
@@ -16905,12 +16908,12 @@
       <c r="D7" s="46" t="n">
         <v>18</v>
       </c>
-      <c r="E7" s="66" t="inlineStr">
+      <c r="E7" s="67" t="inlineStr">
         <is>
           <t>T0409015</t>
         </is>
       </c>
-      <c r="F7" s="65" t="n">
+      <c r="F7" s="66" t="n">
         <v>46314</v>
       </c>
       <c r="G7" s="46" t="n">
@@ -16928,7 +16931,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="65" t="n">
+      <c r="B8" s="66" t="n">
         <v>46314</v>
       </c>
       <c r="C8" s="46" t="n">
@@ -16937,12 +16940,12 @@
       <c r="D8" s="46" t="n">
         <v>18</v>
       </c>
-      <c r="E8" s="66" t="inlineStr">
+      <c r="E8" s="67" t="inlineStr">
         <is>
           <t>T0409016</t>
         </is>
       </c>
-      <c r="F8" s="65" t="n">
+      <c r="F8" s="66" t="n">
         <v>46315</v>
       </c>
       <c r="G8" s="46" t="n">
@@ -16961,7 +16964,7 @@
     </row>
     <row r="9"/>
     <row r="10">
-      <c r="B10" s="57" t="inlineStr">
+      <c r="B10" s="58" t="inlineStr">
         <is>
           <t>TB_R_PRA_DAILY_ORDER_PART</t>
         </is>
@@ -17030,7 +17033,7 @@
           <t>0001</t>
         </is>
       </c>
-      <c r="E12" s="66" t="inlineStr">
+      <c r="E12" s="67" t="inlineStr">
         <is>
           <t>T0409011</t>
         </is>
@@ -17048,7 +17051,7 @@
       <c r="H12" s="46" t="n">
         <v>12</v>
       </c>
-      <c r="I12" s="65" t="n">
+      <c r="I12" s="66" t="n">
         <v>46311</v>
       </c>
       <c r="J12" s="46" t="inlineStr">
@@ -17073,7 +17076,7 @@
           <t>0001</t>
         </is>
       </c>
-      <c r="E13" s="66" t="inlineStr">
+      <c r="E13" s="67" t="inlineStr">
         <is>
           <t>T0409012</t>
         </is>
@@ -17091,7 +17094,7 @@
       <c r="H13" s="46" t="n">
         <v>6</v>
       </c>
-      <c r="I13" s="65" t="n">
+      <c r="I13" s="66" t="n">
         <v>46312</v>
       </c>
       <c r="J13" s="46" t="inlineStr">
@@ -17116,7 +17119,7 @@
           <t>0001</t>
         </is>
       </c>
-      <c r="E14" s="66" t="inlineStr">
+      <c r="E14" s="67" t="inlineStr">
         <is>
           <t>T0409013</t>
         </is>
@@ -17131,10 +17134,10 @@
           <t>PART-X</t>
         </is>
       </c>
-      <c r="H14" s="59" t="n">
+      <c r="H14" s="60" t="n">
         <v>18</v>
       </c>
-      <c r="I14" s="65" t="n">
+      <c r="I14" s="66" t="n">
         <v>46313</v>
       </c>
       <c r="J14" s="46" t="inlineStr">
@@ -17159,7 +17162,7 @@
           <t>0001</t>
         </is>
       </c>
-      <c r="E15" s="67" t="inlineStr">
+      <c r="E15" s="68" t="inlineStr">
         <is>
           <t>T0409014</t>
         </is>
@@ -17177,7 +17180,7 @@
       <c r="H15" s="46" t="n">
         <v>12</v>
       </c>
-      <c r="I15" s="65" t="n">
+      <c r="I15" s="66" t="n">
         <v>46314</v>
       </c>
       <c r="J15" s="46" t="inlineStr">
@@ -17202,7 +17205,7 @@
           <t>0001</t>
         </is>
       </c>
-      <c r="E16" s="66" t="inlineStr">
+      <c r="E16" s="67" t="inlineStr">
         <is>
           <t>T0409015</t>
         </is>
@@ -17220,7 +17223,7 @@
       <c r="H16" s="46" t="n">
         <v>18</v>
       </c>
-      <c r="I16" s="65" t="n">
+      <c r="I16" s="66" t="n">
         <v>46314</v>
       </c>
       <c r="J16" s="46" t="inlineStr">
@@ -17245,7 +17248,7 @@
           <t>0001</t>
         </is>
       </c>
-      <c r="E17" s="66" t="inlineStr">
+      <c r="E17" s="67" t="inlineStr">
         <is>
           <t>T0409016</t>
         </is>
@@ -17263,7 +17266,7 @@
       <c r="H17" s="46" t="n">
         <v>18</v>
       </c>
-      <c r="I17" s="65" t="n">
+      <c r="I17" s="66" t="n">
         <v>46315</v>
       </c>
       <c r="J17" s="46" t="inlineStr">
@@ -17274,7 +17277,7 @@
     </row>
     <row r="18"/>
     <row r="19">
-      <c r="B19" s="57" t="inlineStr">
+      <c r="B19" s="58" t="inlineStr">
         <is>
           <t>TB_R_PRA_DAILY_ORDER_MAPPED</t>
         </is>
@@ -17328,12 +17331,12 @@
           <t>17/10/2026</t>
         </is>
       </c>
-      <c r="C21" s="66" t="inlineStr">
+      <c r="C21" s="67" t="inlineStr">
         <is>
           <t>T0409011</t>
         </is>
       </c>
-      <c r="D21" s="66" t="inlineStr">
+      <c r="D21" s="67" t="inlineStr">
         <is>
           <t>3126035911</t>
         </is>
@@ -17366,12 +17369,12 @@
           <t>18/10/2026</t>
         </is>
       </c>
-      <c r="C22" s="66" t="inlineStr">
+      <c r="C22" s="67" t="inlineStr">
         <is>
           <t>T0409012</t>
         </is>
       </c>
-      <c r="D22" s="66" t="inlineStr">
+      <c r="D22" s="67" t="inlineStr">
         <is>
           <t>3126035912</t>
         </is>
@@ -17404,12 +17407,12 @@
           <t>18/10/2026</t>
         </is>
       </c>
-      <c r="C23" s="66" t="inlineStr">
+      <c r="C23" s="67" t="inlineStr">
         <is>
           <t>T0409013</t>
         </is>
       </c>
-      <c r="D23" s="66" t="inlineStr">
+      <c r="D23" s="67" t="inlineStr">
         <is>
           <t>3126035913</t>
         </is>
@@ -17442,12 +17445,12 @@
           <t>19/10/2026</t>
         </is>
       </c>
-      <c r="C24" s="66" t="inlineStr">
+      <c r="C24" s="67" t="inlineStr">
         <is>
           <t>T0409014</t>
         </is>
       </c>
-      <c r="D24" s="66" t="inlineStr">
+      <c r="D24" s="67" t="inlineStr">
         <is>
           <t>3126035914</t>
         </is>
@@ -17480,12 +17483,12 @@
           <t>20/10/2026</t>
         </is>
       </c>
-      <c r="C25" s="66" t="inlineStr">
+      <c r="C25" s="67" t="inlineStr">
         <is>
           <t>T0409015</t>
         </is>
       </c>
-      <c r="D25" s="66" t="inlineStr">
+      <c r="D25" s="67" t="inlineStr">
         <is>
           <t>3126035915</t>
         </is>
@@ -17518,12 +17521,12 @@
           <t>20/10/2026</t>
         </is>
       </c>
-      <c r="C26" s="66" t="inlineStr">
+      <c r="C26" s="67" t="inlineStr">
         <is>
           <t>T0409016</t>
         </is>
       </c>
-      <c r="D26" s="66" t="inlineStr">
+      <c r="D26" s="67" t="inlineStr">
         <is>
           <t>3126035916</t>
         </is>
@@ -17552,7 +17555,7 @@
     </row>
     <row r="27"/>
     <row r="28">
-      <c r="B28" s="57" t="inlineStr">
+      <c r="B28" s="58" t="inlineStr">
         <is>
           <t>TB_R_INSTRUCTION</t>
         </is>
@@ -17685,12 +17688,12 @@
           <t>9715300</t>
         </is>
       </c>
-      <c r="I30" s="66" t="inlineStr">
+      <c r="I30" s="67" t="inlineStr">
         <is>
           <t>CO-14101</t>
         </is>
       </c>
-      <c r="J30" s="65" t="n">
+      <c r="J30" s="66" t="n">
         <v>46310</v>
       </c>
       <c r="K30" s="46" t="inlineStr">
@@ -17711,12 +17714,12 @@
       <c r="N30" s="46" t="n">
         <v>6</v>
       </c>
-      <c r="O30" s="66" t="inlineStr">
+      <c r="O30" s="67" t="inlineStr">
         <is>
           <t>T0409011</t>
         </is>
       </c>
-      <c r="P30" s="66" t="inlineStr">
+      <c r="P30" s="67" t="inlineStr">
         <is>
           <t>3126035911</t>
         </is>
@@ -17768,12 +17771,12 @@
           <t>9722D10</t>
         </is>
       </c>
-      <c r="I31" s="66" t="inlineStr">
+      <c r="I31" s="67" t="inlineStr">
         <is>
           <t>CO-14103</t>
         </is>
       </c>
-      <c r="J31" s="65" t="n">
+      <c r="J31" s="66" t="n">
         <v>46311</v>
       </c>
       <c r="K31" s="46" t="inlineStr">
@@ -17794,12 +17797,12 @@
       <c r="N31" s="46" t="n">
         <v>6</v>
       </c>
-      <c r="O31" s="66" t="inlineStr">
+      <c r="O31" s="67" t="inlineStr">
         <is>
           <t>T0409011</t>
         </is>
       </c>
-      <c r="P31" s="66" t="inlineStr">
+      <c r="P31" s="67" t="inlineStr">
         <is>
           <t>3126035911</t>
         </is>
@@ -17855,12 +17858,12 @@
           <t>9715300</t>
         </is>
       </c>
-      <c r="I32" s="66" t="inlineStr">
+      <c r="I32" s="67" t="inlineStr">
         <is>
           <t>CO-14105</t>
         </is>
       </c>
-      <c r="J32" s="65" t="n">
+      <c r="J32" s="66" t="n">
         <v>46312</v>
       </c>
       <c r="K32" s="46" t="inlineStr">
@@ -17881,12 +17884,12 @@
       <c r="N32" s="46" t="n">
         <v>6</v>
       </c>
-      <c r="O32" s="66" t="inlineStr">
+      <c r="O32" s="67" t="inlineStr">
         <is>
           <t>T0409012</t>
         </is>
       </c>
-      <c r="P32" s="66" t="inlineStr">
+      <c r="P32" s="67" t="inlineStr">
         <is>
           <t>3126035912</t>
         </is>
@@ -17942,12 +17945,12 @@
           <t>9715300</t>
         </is>
       </c>
-      <c r="I33" s="66" t="inlineStr">
+      <c r="I33" s="67" t="inlineStr">
         <is>
           <t>CO-14106</t>
         </is>
       </c>
-      <c r="J33" s="65" t="n">
+      <c r="J33" s="66" t="n">
         <v>46312</v>
       </c>
       <c r="K33" s="46" t="inlineStr">
@@ -17968,12 +17971,12 @@
       <c r="N33" s="46" t="n">
         <v>3</v>
       </c>
-      <c r="O33" s="66" t="inlineStr">
+      <c r="O33" s="67" t="inlineStr">
         <is>
           <t>T0409013</t>
         </is>
       </c>
-      <c r="P33" s="66" t="inlineStr">
+      <c r="P33" s="67" t="inlineStr">
         <is>
           <t>3126035913</t>
         </is>
@@ -18025,12 +18028,12 @@
           <t>9715300</t>
         </is>
       </c>
-      <c r="I34" s="66" t="inlineStr">
+      <c r="I34" s="67" t="inlineStr">
         <is>
           <t>CO-14107</t>
         </is>
       </c>
-      <c r="J34" s="65" t="n">
+      <c r="J34" s="66" t="n">
         <v>46312</v>
       </c>
       <c r="K34" s="46" t="inlineStr">
@@ -18051,12 +18054,12 @@
       <c r="N34" s="46" t="n">
         <v>3</v>
       </c>
-      <c r="O34" s="66" t="inlineStr">
+      <c r="O34" s="67" t="inlineStr">
         <is>
           <t>T0409013</t>
         </is>
       </c>
-      <c r="P34" s="66" t="inlineStr">
+      <c r="P34" s="67" t="inlineStr">
         <is>
           <t>3126035913</t>
         </is>
@@ -18112,12 +18115,12 @@
           <t>9722D10</t>
         </is>
       </c>
-      <c r="I35" s="66" t="inlineStr">
+      <c r="I35" s="67" t="inlineStr">
         <is>
           <t>CO-14104</t>
         </is>
       </c>
-      <c r="J35" s="65" t="n">
+      <c r="J35" s="66" t="n">
         <v>46312</v>
       </c>
       <c r="K35" s="46" t="inlineStr">
@@ -18138,12 +18141,12 @@
       <c r="N35" s="46" t="n">
         <v>6</v>
       </c>
-      <c r="O35" s="66" t="inlineStr">
+      <c r="O35" s="67" t="inlineStr">
         <is>
           <t>T0409013</t>
         </is>
       </c>
-      <c r="P35" s="66" t="inlineStr">
+      <c r="P35" s="67" t="inlineStr">
         <is>
           <t>3126035913</t>
         </is>
@@ -18199,12 +18202,12 @@
           <t>9811100</t>
         </is>
       </c>
-      <c r="I36" s="66" t="inlineStr">
+      <c r="I36" s="67" t="inlineStr">
         <is>
           <t>CO-14109</t>
         </is>
       </c>
-      <c r="J36" s="65" t="n">
+      <c r="J36" s="66" t="n">
         <v>46312</v>
       </c>
       <c r="K36" s="46" t="inlineStr">
@@ -18225,12 +18228,12 @@
       <c r="N36" s="46" t="n">
         <v>6</v>
       </c>
-      <c r="O36" s="66" t="inlineStr">
+      <c r="O36" s="67" t="inlineStr">
         <is>
           <t>T0409013</t>
         </is>
       </c>
-      <c r="P36" s="66" t="inlineStr">
+      <c r="P36" s="67" t="inlineStr">
         <is>
           <t>3126035913</t>
         </is>
@@ -18282,12 +18285,12 @@
           <t>982200</t>
         </is>
       </c>
-      <c r="I37" s="66" t="inlineStr">
+      <c r="I37" s="67" t="inlineStr">
         <is>
           <t>CO-14110</t>
         </is>
       </c>
-      <c r="J37" s="65" t="n">
+      <c r="J37" s="66" t="n">
         <v>46312</v>
       </c>
       <c r="K37" s="46" t="inlineStr">
@@ -18308,12 +18311,12 @@
       <c r="N37" s="46" t="n">
         <v>6</v>
       </c>
-      <c r="O37" s="66" t="inlineStr">
+      <c r="O37" s="67" t="inlineStr">
         <is>
           <t>T0409014</t>
         </is>
       </c>
-      <c r="P37" s="66" t="inlineStr">
+      <c r="P37" s="67" t="inlineStr">
         <is>
           <t>3126035914</t>
         </is>
@@ -18369,12 +18372,12 @@
           <t>9715300</t>
         </is>
       </c>
-      <c r="I38" s="66" t="inlineStr">
+      <c r="I38" s="67" t="inlineStr">
         <is>
           <t>CO-14112</t>
         </is>
       </c>
-      <c r="J38" s="65" t="n">
+      <c r="J38" s="66" t="n">
         <v>46313</v>
       </c>
       <c r="K38" s="46" t="inlineStr">
@@ -18395,12 +18398,12 @@
       <c r="N38" s="46" t="n">
         <v>6</v>
       </c>
-      <c r="O38" s="66" t="inlineStr">
+      <c r="O38" s="67" t="inlineStr">
         <is>
           <t>T0409014</t>
         </is>
       </c>
-      <c r="P38" s="66" t="inlineStr">
+      <c r="P38" s="67" t="inlineStr">
         <is>
           <t>3126035914</t>
         </is>
@@ -18456,12 +18459,12 @@
           <t>9811100</t>
         </is>
       </c>
-      <c r="I39" s="66" t="inlineStr">
+      <c r="I39" s="67" t="inlineStr">
         <is>
           <t>CO-14113</t>
         </is>
       </c>
-      <c r="J39" s="65" t="n">
+      <c r="J39" s="66" t="n">
         <v>46313</v>
       </c>
       <c r="K39" s="46" t="inlineStr">
@@ -18482,12 +18485,12 @@
       <c r="N39" s="46" t="n">
         <v>6</v>
       </c>
-      <c r="O39" s="66" t="inlineStr">
+      <c r="O39" s="67" t="inlineStr">
         <is>
           <t>T0409015</t>
         </is>
       </c>
-      <c r="P39" s="66" t="inlineStr">
+      <c r="P39" s="67" t="inlineStr">
         <is>
           <t>3126035915</t>
         </is>
@@ -18539,12 +18542,12 @@
           <t>982200</t>
         </is>
       </c>
-      <c r="I40" s="66" t="inlineStr">
+      <c r="I40" s="67" t="inlineStr">
         <is>
           <t>CO-14114</t>
         </is>
       </c>
-      <c r="J40" s="65" t="n">
+      <c r="J40" s="66" t="n">
         <v>46313</v>
       </c>
       <c r="K40" s="46" t="inlineStr">
@@ -18565,12 +18568,12 @@
       <c r="N40" s="46" t="n">
         <v>6</v>
       </c>
-      <c r="O40" s="66" t="inlineStr">
+      <c r="O40" s="67" t="inlineStr">
         <is>
           <t>T0409015</t>
         </is>
       </c>
-      <c r="P40" s="66" t="inlineStr">
+      <c r="P40" s="67" t="inlineStr">
         <is>
           <t>3126035915</t>
         </is>
@@ -18622,12 +18625,12 @@
           <t>9715300</t>
         </is>
       </c>
-      <c r="I41" s="66" t="inlineStr">
+      <c r="I41" s="67" t="inlineStr">
         <is>
           <t>CO-14115</t>
         </is>
       </c>
-      <c r="J41" s="65" t="n">
+      <c r="J41" s="66" t="n">
         <v>46314</v>
       </c>
       <c r="K41" s="46" t="inlineStr">
@@ -18648,12 +18651,12 @@
       <c r="N41" s="46" t="n">
         <v>6</v>
       </c>
-      <c r="O41" s="66" t="inlineStr">
+      <c r="O41" s="67" t="inlineStr">
         <is>
           <t>T0409015</t>
         </is>
       </c>
-      <c r="P41" s="66" t="inlineStr">
+      <c r="P41" s="67" t="inlineStr">
         <is>
           <t>3126035915</t>
         </is>
@@ -18714,7 +18717,7 @@
           <t>CO-14115</t>
         </is>
       </c>
-      <c r="J42" s="65" t="n">
+      <c r="J42" s="66" t="n">
         <v>46314</v>
       </c>
       <c r="K42" s="46" t="inlineStr">
@@ -18735,12 +18738,12 @@
       <c r="N42" s="46" t="n">
         <v>6</v>
       </c>
-      <c r="O42" s="66" t="inlineStr">
+      <c r="O42" s="67" t="inlineStr">
         <is>
           <t>T0409016</t>
         </is>
       </c>
-      <c r="P42" s="66" t="inlineStr">
+      <c r="P42" s="67" t="inlineStr">
         <is>
           <t>3126035916</t>
         </is>
@@ -18796,12 +18799,12 @@
           <t>9715300</t>
         </is>
       </c>
-      <c r="I43" s="66" t="inlineStr">
+      <c r="I43" s="67" t="inlineStr">
         <is>
           <t>CO-14115</t>
         </is>
       </c>
-      <c r="J43" s="65" t="n">
+      <c r="J43" s="66" t="n">
         <v>46314</v>
       </c>
       <c r="K43" s="46" t="inlineStr">
@@ -18814,7 +18817,7 @@
           <t>001</t>
         </is>
       </c>
-      <c r="M43" s="60" t="inlineStr">
+      <c r="M43" s="61" t="inlineStr">
         <is>
           <t>0000002</t>
         </is>
@@ -18822,12 +18825,12 @@
       <c r="N43" s="46" t="n">
         <v>6</v>
       </c>
-      <c r="O43" s="66" t="inlineStr">
+      <c r="O43" s="67" t="inlineStr">
         <is>
           <t>T0409016</t>
         </is>
       </c>
-      <c r="P43" s="66" t="inlineStr">
+      <c r="P43" s="67" t="inlineStr">
         <is>
           <t>3126035916</t>
         </is>
@@ -18883,12 +18886,12 @@
           <t>9722D10</t>
         </is>
       </c>
-      <c r="I44" s="68" t="inlineStr">
+      <c r="I44" s="69" t="inlineStr">
         <is>
           <t>CO-14111</t>
         </is>
       </c>
-      <c r="J44" s="69" t="n">
+      <c r="J44" s="70" t="n">
         <v>46314</v>
       </c>
       <c r="K44" s="46" t="inlineStr">
@@ -18909,12 +18912,12 @@
       <c r="N44" s="46" t="n">
         <v>6</v>
       </c>
-      <c r="O44" s="66" t="inlineStr">
+      <c r="O44" s="67" t="inlineStr">
         <is>
           <t>T0409013</t>
         </is>
       </c>
-      <c r="P44" s="66" t="inlineStr">
+      <c r="P44" s="67" t="inlineStr">
         <is>
           <t>3126035913</t>
         </is>
@@ -18942,7 +18945,7 @@
     </row>
     <row r="45"/>
     <row r="46">
-      <c r="B46" s="57" t="inlineStr">
+      <c r="B46" s="58" t="inlineStr">
         <is>
           <t>TB_H_CROSSDOCK_ORDER_CHANGE</t>
         </is>
@@ -19024,7 +19027,7 @@
       <c r="C48" s="46" t="n">
         <v>1</v>
       </c>
-      <c r="D48" s="66" t="inlineStr">
+      <c r="D48" s="67" t="inlineStr">
         <is>
           <t>ASN0003</t>
         </is>
@@ -19039,7 +19042,7 @@
           <t>PART-X</t>
         </is>
       </c>
-      <c r="G48" s="66" t="inlineStr">
+      <c r="G48" s="67" t="inlineStr">
         <is>
           <t>CO-14104</t>
         </is>
@@ -19049,7 +19052,7 @@
           <t>0000001</t>
         </is>
       </c>
-      <c r="I48" s="66" t="inlineStr">
+      <c r="I48" s="67" t="inlineStr">
         <is>
           <t>CO-14111</t>
         </is>
@@ -19062,10 +19065,10 @@
       <c r="K48" s="46" t="n">
         <v>6</v>
       </c>
-      <c r="L48" s="66" t="n">
-        <v>6</v>
-      </c>
-      <c r="M48" s="66" t="n">
+      <c r="L48" s="67" t="n">
+        <v>6</v>
+      </c>
+      <c r="M48" s="67" t="n">
         <v>6</v>
       </c>
       <c r="N48" s="46" t="inlineStr">
@@ -19184,14 +19187,14 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="62" t="inlineStr">
+      <c r="A1" s="63" t="inlineStr">
         <is>
           <t>Hasil XD09 [Search] per hari. PART-X 6 pcs/case. Urutan = ORDER_DT (Allocation Priority), CUSTOMER_CD, CUSTOMER_ORDER_NO, ...; PO urut PO_DT (sisa open qty). Hanya line UPDT_STATUS NULL, HOLD_FLAG N, PO_MAPPED_FLAG N. GROUP_SEQ hanya logic.</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="70" t="inlineStr">
+      <c r="A2" s="71" t="inlineStr">
         <is>
           <t>Teks biru bergaris bawah = hyperlink ke tabel terkait (PO_NO / MANIFEST_NO → TB_R_PRA_DAILY_ORDER_PART, CUSTOMER_ORDER_NO → H0253 replicate di Sheet1).</t>
         </is>
@@ -19199,7 +19202,7 @@
     </row>
     <row r="3"/>
     <row r="4">
-      <c r="A4" s="57" t="inlineStr">
+      <c r="A4" s="58" t="inlineStr">
         <is>
           <t>16/10/2026 [Search] (CO-14102 Hold → tidak diambil)</t>
         </is>
@@ -19301,7 +19304,7 @@
           <t>PART-X</t>
         </is>
       </c>
-      <c r="C6" s="65" t="n">
+      <c r="C6" s="66" t="n">
         <v>46310</v>
       </c>
       <c r="D6" s="46" t="inlineStr">
@@ -19309,7 +19312,7 @@
           <t>9715300</t>
         </is>
       </c>
-      <c r="E6" s="66" t="inlineStr">
+      <c r="E6" s="67" t="inlineStr">
         <is>
           <t>CO-14101</t>
         </is>
@@ -19325,12 +19328,12 @@
       <c r="H6" s="46" t="n">
         <v>6</v>
       </c>
-      <c r="I6" s="66" t="inlineStr">
+      <c r="I6" s="67" t="inlineStr">
         <is>
           <t>T0409011</t>
         </is>
       </c>
-      <c r="J6" s="66" t="inlineStr">
+      <c r="J6" s="67" t="inlineStr">
         <is>
           <t>3126035911</t>
         </is>
@@ -19344,7 +19347,7 @@
       <c r="M6" s="46" t="n">
         <v>6</v>
       </c>
-      <c r="N6" s="60" t="inlineStr">
+      <c r="N6" s="61" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -19365,7 +19368,7 @@
     </row>
     <row r="7"/>
     <row r="8">
-      <c r="A8" s="57" t="inlineStr">
+      <c r="A8" s="58" t="inlineStr">
         <is>
           <t>17/10/2026 [Search]</t>
         </is>
@@ -19467,7 +19470,7 @@
           <t>PART-X</t>
         </is>
       </c>
-      <c r="C10" s="65" t="n">
+      <c r="C10" s="66" t="n">
         <v>46311</v>
       </c>
       <c r="D10" s="46" t="inlineStr">
@@ -19475,7 +19478,7 @@
           <t>9722D10</t>
         </is>
       </c>
-      <c r="E10" s="66" t="inlineStr">
+      <c r="E10" s="67" t="inlineStr">
         <is>
           <t>CO-14103</t>
         </is>
@@ -19491,12 +19494,12 @@
       <c r="H10" s="46" t="n">
         <v>6</v>
       </c>
-      <c r="I10" s="66" t="inlineStr">
+      <c r="I10" s="67" t="inlineStr">
         <is>
           <t>T0409011</t>
         </is>
       </c>
-      <c r="J10" s="66" t="inlineStr">
+      <c r="J10" s="67" t="inlineStr">
         <is>
           <t>3126035911</t>
         </is>
@@ -19510,7 +19513,7 @@
       <c r="M10" s="46" t="n">
         <v>6</v>
       </c>
-      <c r="N10" s="60" t="inlineStr">
+      <c r="N10" s="61" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -19531,7 +19534,7 @@
     </row>
     <row r="11"/>
     <row r="12">
-      <c r="A12" s="57" t="inlineStr">
+      <c r="A12" s="58" t="inlineStr">
         <is>
           <t>18/10/2026 [Search]: order date 17/10, 4 destinasi, PO tersedia 24 dari 30 (abnormal)</t>
         </is>
@@ -19633,7 +19636,7 @@
           <t>PART-X</t>
         </is>
       </c>
-      <c r="C14" s="65" t="n">
+      <c r="C14" s="66" t="n">
         <v>46312</v>
       </c>
       <c r="D14" s="46" t="inlineStr">
@@ -19641,7 +19644,7 @@
           <t>9715300</t>
         </is>
       </c>
-      <c r="E14" s="66" t="inlineStr">
+      <c r="E14" s="67" t="inlineStr">
         <is>
           <t>CO-14105</t>
         </is>
@@ -19657,12 +19660,12 @@
       <c r="H14" s="46" t="n">
         <v>6</v>
       </c>
-      <c r="I14" s="66" t="inlineStr">
+      <c r="I14" s="67" t="inlineStr">
         <is>
           <t>T0409012</t>
         </is>
       </c>
-      <c r="J14" s="66" t="inlineStr">
+      <c r="J14" s="67" t="inlineStr">
         <is>
           <t>3126035912</t>
         </is>
@@ -19676,7 +19679,7 @@
       <c r="M14" s="46" t="n">
         <v>6</v>
       </c>
-      <c r="N14" s="60" t="inlineStr">
+      <c r="N14" s="61" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -19704,7 +19707,7 @@
           <t>PART-X</t>
         </is>
       </c>
-      <c r="C15" s="65" t="n">
+      <c r="C15" s="66" t="n">
         <v>46312</v>
       </c>
       <c r="D15" s="46" t="inlineStr">
@@ -19712,7 +19715,7 @@
           <t>9715300</t>
         </is>
       </c>
-      <c r="E15" s="66" t="inlineStr">
+      <c r="E15" s="67" t="inlineStr">
         <is>
           <t>CO-14106</t>
         </is>
@@ -19728,12 +19731,12 @@
       <c r="H15" s="46" t="n">
         <v>3</v>
       </c>
-      <c r="I15" s="66" t="inlineStr">
+      <c r="I15" s="67" t="inlineStr">
         <is>
           <t>T0409013</t>
         </is>
       </c>
-      <c r="J15" s="66" t="inlineStr">
+      <c r="J15" s="67" t="inlineStr">
         <is>
           <t>3126035913</t>
         </is>
@@ -19771,7 +19774,7 @@
           <t>PART-X</t>
         </is>
       </c>
-      <c r="C16" s="65" t="n">
+      <c r="C16" s="66" t="n">
         <v>46312</v>
       </c>
       <c r="D16" s="46" t="inlineStr">
@@ -19779,7 +19782,7 @@
           <t>9715300</t>
         </is>
       </c>
-      <c r="E16" s="66" t="inlineStr">
+      <c r="E16" s="67" t="inlineStr">
         <is>
           <t>CO-14107</t>
         </is>
@@ -19795,12 +19798,12 @@
       <c r="H16" s="46" t="n">
         <v>3</v>
       </c>
-      <c r="I16" s="66" t="inlineStr">
+      <c r="I16" s="67" t="inlineStr">
         <is>
           <t>T0409013</t>
         </is>
       </c>
-      <c r="J16" s="66" t="inlineStr">
+      <c r="J16" s="67" t="inlineStr">
         <is>
           <t>3126035913</t>
         </is>
@@ -19814,7 +19817,7 @@
       <c r="M16" s="46" t="n">
         <v>6</v>
       </c>
-      <c r="N16" s="60" t="inlineStr">
+      <c r="N16" s="61" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -19838,7 +19841,7 @@
           <t>PART-X</t>
         </is>
       </c>
-      <c r="C17" s="65" t="n">
+      <c r="C17" s="66" t="n">
         <v>46312</v>
       </c>
       <c r="D17" s="46" t="inlineStr">
@@ -19846,7 +19849,7 @@
           <t>9722D10</t>
         </is>
       </c>
-      <c r="E17" s="66" t="inlineStr">
+      <c r="E17" s="67" t="inlineStr">
         <is>
           <t>CO-14104</t>
         </is>
@@ -19862,12 +19865,12 @@
       <c r="H17" s="46" t="n">
         <v>6</v>
       </c>
-      <c r="I17" s="66" t="inlineStr">
+      <c r="I17" s="67" t="inlineStr">
         <is>
           <t>T0409013</t>
         </is>
       </c>
-      <c r="J17" s="66" t="inlineStr">
+      <c r="J17" s="67" t="inlineStr">
         <is>
           <t>3126035913</t>
         </is>
@@ -19881,7 +19884,7 @@
       <c r="M17" s="46" t="n">
         <v>6</v>
       </c>
-      <c r="N17" s="60" t="inlineStr">
+      <c r="N17" s="61" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -19909,7 +19912,7 @@
           <t>PART-X</t>
         </is>
       </c>
-      <c r="C18" s="65" t="n">
+      <c r="C18" s="66" t="n">
         <v>46312</v>
       </c>
       <c r="D18" s="46" t="inlineStr">
@@ -19917,7 +19920,7 @@
           <t>9811100</t>
         </is>
       </c>
-      <c r="E18" s="66" t="inlineStr">
+      <c r="E18" s="67" t="inlineStr">
         <is>
           <t>CO-14109</t>
         </is>
@@ -19933,12 +19936,12 @@
       <c r="H18" s="46" t="n">
         <v>6</v>
       </c>
-      <c r="I18" s="66" t="inlineStr">
+      <c r="I18" s="67" t="inlineStr">
         <is>
           <t>T0409013</t>
         </is>
       </c>
-      <c r="J18" s="66" t="inlineStr">
+      <c r="J18" s="67" t="inlineStr">
         <is>
           <t>3126035913</t>
         </is>
@@ -19952,7 +19955,7 @@
       <c r="M18" s="46" t="n">
         <v>6</v>
       </c>
-      <c r="N18" s="60" t="inlineStr">
+      <c r="N18" s="61" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -19976,7 +19979,7 @@
           <t>PART-X</t>
         </is>
       </c>
-      <c r="C19" s="65" t="n">
+      <c r="C19" s="66" t="n">
         <v>46312</v>
       </c>
       <c r="D19" s="46" t="inlineStr">
@@ -19984,7 +19987,7 @@
           <t>982200</t>
         </is>
       </c>
-      <c r="E19" s="66" t="inlineStr">
+      <c r="E19" s="67" t="inlineStr">
         <is>
           <t>CO-14110</t>
         </is>
@@ -20011,7 +20014,7 @@
       <c r="M19" s="46" t="n">
         <v>6</v>
       </c>
-      <c r="N19" s="60" t="inlineStr">
+      <c r="N19" s="61" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -20019,7 +20022,7 @@
       <c r="O19" s="46" t="n">
         <v>5</v>
       </c>
-      <c r="P19" s="59" t="inlineStr">
+      <c r="P19" s="60" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -20032,7 +20035,7 @@
     </row>
     <row r="20"/>
     <row r="21">
-      <c r="A21" s="57" t="inlineStr">
+      <c r="A21" s="58" t="inlineStr">
         <is>
           <t>19/10/2026 [Search]: sisa order date 17/10 (CO-14104 UPDT 2, Case 1-4 sudah ASN → tidak diambil) + order date 18/10 (3 destinasi)</t>
         </is>
@@ -20134,7 +20137,7 @@
           <t>PART-X</t>
         </is>
       </c>
-      <c r="C23" s="65" t="n">
+      <c r="C23" s="66" t="n">
         <v>46312</v>
       </c>
       <c r="D23" s="46" t="inlineStr">
@@ -20142,7 +20145,7 @@
           <t>982200</t>
         </is>
       </c>
-      <c r="E23" s="66" t="inlineStr">
+      <c r="E23" s="67" t="inlineStr">
         <is>
           <t>CO-14110</t>
         </is>
@@ -20158,12 +20161,12 @@
       <c r="H23" s="46" t="n">
         <v>6</v>
       </c>
-      <c r="I23" s="66" t="inlineStr">
+      <c r="I23" s="67" t="inlineStr">
         <is>
           <t>T0409014</t>
         </is>
       </c>
-      <c r="J23" s="66" t="inlineStr">
+      <c r="J23" s="67" t="inlineStr">
         <is>
           <t>3126035914</t>
         </is>
@@ -20177,7 +20180,7 @@
       <c r="M23" s="46" t="n">
         <v>6</v>
       </c>
-      <c r="N23" s="60" t="inlineStr">
+      <c r="N23" s="61" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -20205,7 +20208,7 @@
           <t>PART-X</t>
         </is>
       </c>
-      <c r="C24" s="65" t="n">
+      <c r="C24" s="66" t="n">
         <v>46313</v>
       </c>
       <c r="D24" s="46" t="inlineStr">
@@ -20213,7 +20216,7 @@
           <t>9715300</t>
         </is>
       </c>
-      <c r="E24" s="66" t="inlineStr">
+      <c r="E24" s="67" t="inlineStr">
         <is>
           <t>CO-14112</t>
         </is>
@@ -20229,12 +20232,12 @@
       <c r="H24" s="46" t="n">
         <v>6</v>
       </c>
-      <c r="I24" s="66" t="inlineStr">
+      <c r="I24" s="67" t="inlineStr">
         <is>
           <t>T0409014</t>
         </is>
       </c>
-      <c r="J24" s="66" t="inlineStr">
+      <c r="J24" s="67" t="inlineStr">
         <is>
           <t>3126035914</t>
         </is>
@@ -20248,7 +20251,7 @@
       <c r="M24" s="46" t="n">
         <v>6</v>
       </c>
-      <c r="N24" s="60" t="inlineStr">
+      <c r="N24" s="61" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -20276,7 +20279,7 @@
           <t>PART-X</t>
         </is>
       </c>
-      <c r="C25" s="65" t="n">
+      <c r="C25" s="66" t="n">
         <v>46313</v>
       </c>
       <c r="D25" s="46" t="inlineStr">
@@ -20284,7 +20287,7 @@
           <t>9811100</t>
         </is>
       </c>
-      <c r="E25" s="66" t="inlineStr">
+      <c r="E25" s="67" t="inlineStr">
         <is>
           <t>CO-14113</t>
         </is>
@@ -20300,12 +20303,12 @@
       <c r="H25" s="46" t="n">
         <v>6</v>
       </c>
-      <c r="I25" s="66" t="inlineStr">
+      <c r="I25" s="67" t="inlineStr">
         <is>
           <t>T0409015</t>
         </is>
       </c>
-      <c r="J25" s="66" t="inlineStr">
+      <c r="J25" s="67" t="inlineStr">
         <is>
           <t>3126035915</t>
         </is>
@@ -20319,7 +20322,7 @@
       <c r="M25" s="46" t="n">
         <v>6</v>
       </c>
-      <c r="N25" s="60" t="inlineStr">
+      <c r="N25" s="61" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -20343,7 +20346,7 @@
           <t>PART-X</t>
         </is>
       </c>
-      <c r="C26" s="65" t="n">
+      <c r="C26" s="66" t="n">
         <v>46313</v>
       </c>
       <c r="D26" s="46" t="inlineStr">
@@ -20351,7 +20354,7 @@
           <t>982200</t>
         </is>
       </c>
-      <c r="E26" s="66" t="inlineStr">
+      <c r="E26" s="67" t="inlineStr">
         <is>
           <t>CO-14114</t>
         </is>
@@ -20367,12 +20370,12 @@
       <c r="H26" s="46" t="n">
         <v>6</v>
       </c>
-      <c r="I26" s="66" t="inlineStr">
+      <c r="I26" s="67" t="inlineStr">
         <is>
           <t>T0409015</t>
         </is>
       </c>
-      <c r="J26" s="66" t="inlineStr">
+      <c r="J26" s="67" t="inlineStr">
         <is>
           <t>3126035915</t>
         </is>
@@ -20386,7 +20389,7 @@
       <c r="M26" s="46" t="n">
         <v>6</v>
       </c>
-      <c r="N26" s="60" t="inlineStr">
+      <c r="N26" s="61" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -20407,7 +20410,7 @@
     </row>
     <row r="27"/>
     <row r="28">
-      <c r="A28" s="57" t="inlineStr">
+      <c r="A28" s="58" t="inlineStr">
         <is>
           <t>20/10/2026 [Search]: order date 19/10 (CO-14115 VN 12 = 2 case, CO-14111 TH 6)</t>
         </is>
@@ -20509,7 +20512,7 @@
           <t>PART-X</t>
         </is>
       </c>
-      <c r="C30" s="65" t="n">
+      <c r="C30" s="66" t="n">
         <v>46314</v>
       </c>
       <c r="D30" s="46" t="inlineStr">
@@ -20517,7 +20520,7 @@
           <t>9715300</t>
         </is>
       </c>
-      <c r="E30" s="66" t="inlineStr">
+      <c r="E30" s="67" t="inlineStr">
         <is>
           <t>CO-14115</t>
         </is>
@@ -20533,12 +20536,12 @@
       <c r="H30" s="46" t="n">
         <v>6</v>
       </c>
-      <c r="I30" s="66" t="inlineStr">
+      <c r="I30" s="67" t="inlineStr">
         <is>
           <t>T0409015</t>
         </is>
       </c>
-      <c r="J30" s="66" t="inlineStr">
+      <c r="J30" s="67" t="inlineStr">
         <is>
           <t>3126035915</t>
         </is>
@@ -20552,7 +20555,7 @@
       <c r="M30" s="46" t="n">
         <v>6</v>
       </c>
-      <c r="N30" s="60" t="inlineStr">
+      <c r="N30" s="61" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -20580,7 +20583,7 @@
           <t>PART-X</t>
         </is>
       </c>
-      <c r="C31" s="65" t="n">
+      <c r="C31" s="66" t="n">
         <v>46314</v>
       </c>
       <c r="D31" s="46" t="inlineStr">
@@ -20588,7 +20591,7 @@
           <t>9715300</t>
         </is>
       </c>
-      <c r="E31" s="66" t="inlineStr">
+      <c r="E31" s="67" t="inlineStr">
         <is>
           <t>CO-14115</t>
         </is>
@@ -20604,12 +20607,12 @@
       <c r="H31" s="46" t="n">
         <v>6</v>
       </c>
-      <c r="I31" s="66" t="inlineStr">
+      <c r="I31" s="67" t="inlineStr">
         <is>
           <t>T0409016</t>
         </is>
       </c>
-      <c r="J31" s="66" t="inlineStr">
+      <c r="J31" s="67" t="inlineStr">
         <is>
           <t>3126035916</t>
         </is>
@@ -20623,7 +20626,7 @@
       <c r="M31" s="46" t="n">
         <v>6</v>
       </c>
-      <c r="N31" s="60" t="inlineStr">
+      <c r="N31" s="61" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -20651,7 +20654,7 @@
           <t>PART-X</t>
         </is>
       </c>
-      <c r="C32" s="65" t="n">
+      <c r="C32" s="66" t="n">
         <v>46314</v>
       </c>
       <c r="D32" s="46" t="inlineStr">
@@ -20659,7 +20662,7 @@
           <t>9722D10</t>
         </is>
       </c>
-      <c r="E32" s="66" t="inlineStr">
+      <c r="E32" s="67" t="inlineStr">
         <is>
           <t>CO-14111</t>
         </is>
@@ -20675,12 +20678,12 @@
       <c r="H32" s="46" t="n">
         <v>6</v>
       </c>
-      <c r="I32" s="66" t="inlineStr">
+      <c r="I32" s="67" t="inlineStr">
         <is>
           <t>T0409016</t>
         </is>
       </c>
-      <c r="J32" s="66" t="inlineStr">
+      <c r="J32" s="67" t="inlineStr">
         <is>
           <t>3126035916</t>
         </is>
@@ -20694,7 +20697,7 @@
       <c r="M32" s="46" t="n">
         <v>6</v>
       </c>
-      <c r="N32" s="60" t="inlineStr">
+      <c r="N32" s="61" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -20715,7 +20718,7 @@
     </row>
     <row r="33"/>
     <row r="34">
-      <c r="A34" s="57" t="inlineStr">
+      <c r="A34" s="58" t="inlineStr">
         <is>
           <t>21/10/2026 [Search] SALAH (tanpa tata ulang TB_R_INSTRUCTION): serial 0000002 dianggap open 6 → mapping lagi</t>
         </is>
@@ -20817,7 +20820,7 @@
           <t>PART-X</t>
         </is>
       </c>
-      <c r="C36" s="65" t="n">
+      <c r="C36" s="66" t="n">
         <v>46314</v>
       </c>
       <c r="D36" s="46" t="inlineStr">
@@ -20825,7 +20828,7 @@
           <t>9715300</t>
         </is>
       </c>
-      <c r="E36" s="66" t="inlineStr">
+      <c r="E36" s="67" t="inlineStr">
         <is>
           <t>CO-14115</t>
         </is>
@@ -20841,12 +20844,12 @@
       <c r="H36" s="46" t="n">
         <v>6</v>
       </c>
-      <c r="I36" s="66" t="inlineStr">
+      <c r="I36" s="67" t="inlineStr">
         <is>
           <t>T0409016</t>
         </is>
       </c>
-      <c r="J36" s="66" t="inlineStr">
+      <c r="J36" s="67" t="inlineStr">
         <is>
           <t>3126035916</t>
         </is>
@@ -20860,7 +20863,7 @@
       <c r="M36" s="46" t="n">
         <v>6</v>
       </c>
-      <c r="N36" s="60" t="inlineStr">
+      <c r="N36" s="61" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -20881,14 +20884,14 @@
     </row>
     <row r="37"/>
     <row r="38">
-      <c r="A38" s="62" t="inlineStr">
+      <c r="A38" s="63" t="inlineStr">
         <is>
           <t>21/10/2026 [Search] BENAR (dengan tata ulang XD08): serial 0000001 = ASN0006, serial 0000002 = ASN0007 → open qty 0, tidak ada line diambil. CO-14111 UPDT 6 → tidak diambil; dapat Case 3 ASN0003 lewat Change Order Number.</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="62" t="inlineStr">
+      <c r="A39" s="63" t="inlineStr">
         <is>
           <t>Sisa PO open di akhir: T0409016 12 pcs = qty cancel CO-14102 + CO-14104.</t>
         </is>

</xml_diff>